<commit_message>
New public datasets added
</commit_message>
<xml_diff>
--- a/goldStandard/_Index.xlsx
+++ b/goldStandard/_Index.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julia\Documents\GitHub\normScore\goldStandard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB3DFF11-BAED-4F69-BE87-8051C588F506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A645F18-FB62-4283-832A-F711B021F64D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-22046" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{F827C457-048B-4104-BF2A-59E43A6422D6}"/>
+    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{F827C457-048B-4104-BF2A-59E43A6422D6}"/>
   </bookViews>
   <sheets>
     <sheet name="In" sheetId="1" r:id="rId1"/>
     <sheet name="Out" sheetId="2" r:id="rId2"/>
+    <sheet name="Possible" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="260">
   <si>
     <t>ID</t>
   </si>
@@ -208,9 +209,6 @@
     <t>DOI: 10.1021/ACS.JPROTEOME.3C00677</t>
   </si>
   <si>
-    <t>spectral count todo?</t>
-  </si>
-  <si>
     <t>PXD058626</t>
   </si>
   <si>
@@ -220,9 +218,6 @@
     <t>Lung tissue</t>
   </si>
   <si>
-    <t>Control;IPF</t>
-  </si>
-  <si>
     <t>DOI: 10.1172/JCI.INSIGHT.189636</t>
   </si>
   <si>
@@ -347,6 +342,471 @@
   </si>
   <si>
     <t>From meta-analysis 944 (searching there corresponce between group - samples)</t>
+  </si>
+  <si>
+    <t>Quedan poucas proteínas e teñen formas raras nas gráficas de evaluación… mais que raras, sin forma. Quizás hai que eliminar</t>
+  </si>
+  <si>
+    <t>Control;IPF X Alveoli;Airway;</t>
+  </si>
+  <si>
+    <t>PXD022614</t>
+  </si>
+  <si>
+    <t>LTQ Orbitrap;Q Exactive</t>
+  </si>
+  <si>
+    <t>Adult;Adult+Sperm;Young</t>
+  </si>
+  <si>
+    <t>PXD019504</t>
+  </si>
+  <si>
+    <t>Colon</t>
+  </si>
+  <si>
+    <t>C;T</t>
+  </si>
+  <si>
+    <t>DOI: 10.18632/oncotarget.27491</t>
+  </si>
+  <si>
+    <t>PXD054553</t>
+  </si>
+  <si>
+    <t>Blood</t>
+  </si>
+  <si>
+    <t>BJAB;MEC-1</t>
+  </si>
+  <si>
+    <t>DOI: 10.1016/J.JBC.2025.108386</t>
+  </si>
+  <si>
+    <t>PXD054636</t>
+  </si>
+  <si>
+    <t>Con;VEGFA;BRK</t>
+  </si>
+  <si>
+    <t>PXD054712 for the same author, same illness</t>
+  </si>
+  <si>
+    <t>PXD054817</t>
+  </si>
+  <si>
+    <t>Q Exactive</t>
+  </si>
+  <si>
+    <t>ARIDA;IgG</t>
+  </si>
+  <si>
+    <t>DOI: 10.1002/1878-0261.70019</t>
+  </si>
+  <si>
+    <t>Experiment 1</t>
+  </si>
+  <si>
+    <t>Experiment 2</t>
+  </si>
+  <si>
+    <t>Cntl;IPL</t>
+  </si>
+  <si>
+    <t>PXD054817.2</t>
+  </si>
+  <si>
+    <t>PXD046983</t>
+  </si>
+  <si>
+    <t>ZenoTOF 7600</t>
+  </si>
+  <si>
+    <t>DIANN</t>
+  </si>
+  <si>
+    <t>Retina</t>
+  </si>
+  <si>
+    <t>Ctl;LIM</t>
+  </si>
+  <si>
+    <t>TSV: sample info PXD046983.sdrf.tsv</t>
+  </si>
+  <si>
+    <t>PXD050996</t>
+  </si>
+  <si>
+    <t>Heart</t>
+  </si>
+  <si>
+    <t>CA;CP;MA;MP</t>
+  </si>
+  <si>
+    <t>Group info from sample name | PXD050990 from same research</t>
+  </si>
+  <si>
+    <t>PXD052720</t>
+  </si>
+  <si>
+    <t>Dengue;Control</t>
+  </si>
+  <si>
+    <t>DOI: 10.1002/jmv.29775</t>
+  </si>
+  <si>
+    <t>PXD062678</t>
+  </si>
+  <si>
+    <t>timsTOF Pro 2</t>
+  </si>
+  <si>
+    <t>Saliva</t>
+  </si>
+  <si>
+    <t>Control;OSCC;Premalignant</t>
+  </si>
+  <si>
+    <t>PXD063236</t>
+  </si>
+  <si>
+    <t>Control;Moyamoya</t>
+  </si>
+  <si>
+    <t>PXD063383</t>
+  </si>
+  <si>
+    <t>BV2;EMPTY;SCR;SPI1KD;SPI1OE</t>
+  </si>
+  <si>
+    <t>PXD063923</t>
+  </si>
+  <si>
+    <t>WT;IT;RX</t>
+  </si>
+  <si>
+    <t>DOI: 10.1016/J.MCPRO.2025.101462</t>
+  </si>
+  <si>
+    <t>PXD058791</t>
+  </si>
+  <si>
+    <t>Myc.M.aMum1.;Myc.M.IgG.;Myc.M.aMvc.;Vec.a.MVC.</t>
+  </si>
+  <si>
+    <t>PXD058655</t>
+  </si>
+  <si>
+    <t>Orbitrap Eclipse</t>
+  </si>
+  <si>
+    <t>0h;12h;24h</t>
+  </si>
+  <si>
+    <t>DOI: 10.1101/2023.09.16.558067</t>
+  </si>
+  <si>
+    <t>PXD051732</t>
+  </si>
+  <si>
+    <t>Escherichia coli</t>
+  </si>
+  <si>
+    <t>maXis</t>
+  </si>
+  <si>
+    <t>CI3_M5;CI3_WT;CI23_M3;CI23_WT;CI39_M3;CI39_WT</t>
+  </si>
+  <si>
+    <t>DOI: 10.1038/S44259-024-00050-7</t>
+  </si>
+  <si>
+    <t>PXD047566</t>
+  </si>
+  <si>
+    <t>Same paper PXD051732</t>
+  </si>
+  <si>
+    <t>WT;M3;M6;M8;WT_T;M3_T;M6_T;M8_T</t>
+  </si>
+  <si>
+    <t>PXD055964</t>
+  </si>
+  <si>
+    <t>Aortic tissue</t>
+  </si>
+  <si>
+    <t>WT_No;fl/fl_No;WT_Yes;fl/fl_Yes</t>
+  </si>
+  <si>
+    <t>DOI: 10.1016/j.jbc.2025.108400</t>
+  </si>
+  <si>
+    <t>XLSX: PXD055964_Metadata.xlsx</t>
+  </si>
+  <si>
+    <t>PXD060381</t>
+  </si>
+  <si>
+    <t>Orbitrap Astral</t>
+  </si>
+  <si>
+    <t>WT;NT;TS</t>
+  </si>
+  <si>
+    <t>DOI: 10.1007/s12195-025-00843-4</t>
+  </si>
+  <si>
+    <t>PXD056859</t>
+  </si>
+  <si>
+    <t>Oocyte</t>
+  </si>
+  <si>
+    <t>WT;Het;Hom</t>
+  </si>
+  <si>
+    <t>DOI: 10.1093/molehr/gaaf055</t>
+  </si>
+  <si>
+    <t>PXD047128</t>
+  </si>
+  <si>
+    <t>Urine</t>
+  </si>
+  <si>
+    <t>UW;UO;UP</t>
+  </si>
+  <si>
+    <t>PXD064948</t>
+  </si>
+  <si>
+    <t>Unfixed;fixed</t>
+  </si>
+  <si>
+    <t>DOI: 10.1016/j.ocarto.2025.100664</t>
+  </si>
+  <si>
+    <t>Chondrocytes</t>
+  </si>
+  <si>
+    <t>timsTOF HT</t>
+  </si>
+  <si>
+    <t>PXD051201</t>
+  </si>
+  <si>
+    <t>Men;Women</t>
+  </si>
+  <si>
+    <t>TXT: PXD051201_DM.xlsx</t>
+  </si>
+  <si>
+    <t>DM file created from an additional XLSX in PRIDE and Supplementary Material wit group info</t>
+  </si>
+  <si>
+    <t>DOI: 10.1186/s12014-025-09549-1</t>
+  </si>
+  <si>
+    <t>PXD068597</t>
+  </si>
+  <si>
+    <t>Young;OLD</t>
+  </si>
+  <si>
+    <t>DOI: 10.1158/0008-5472.can-25-1904</t>
+  </si>
+  <si>
+    <t>PXD060921</t>
+  </si>
+  <si>
+    <t>timsTOF fleX</t>
+  </si>
+  <si>
+    <t>Neuronal stem cell</t>
+  </si>
+  <si>
+    <t>EV.VH;NI;PBS;ND</t>
+  </si>
+  <si>
+    <t>DOI: 10.1002/jex2.70108</t>
+  </si>
+  <si>
+    <t>PXD071471</t>
+  </si>
+  <si>
+    <t>AR_3rdT;AH_6MPP;H_3rdT;H_6MPP</t>
+  </si>
+  <si>
+    <t>DOI: 10.1016/J.ARCHORALBIO.2025.106319</t>
+  </si>
+  <si>
+    <t>XLSX: PXD071471_SDRF_pregnancy.xlsx</t>
+  </si>
+  <si>
+    <t>PXD057069</t>
+  </si>
+  <si>
+    <t>WT_CTSB;AD_CTSB;AD_Con;WT_Con</t>
+  </si>
+  <si>
+    <t>DOI: 10.1111/acel.70242</t>
+  </si>
+  <si>
+    <t>TXT: PXD057069_HvP_Metadata.txt</t>
+  </si>
+  <si>
+    <t>There are also quantification files for blood and muscle!</t>
+  </si>
+  <si>
+    <t>PXD055158</t>
+  </si>
+  <si>
+    <t>TripleTOF 5600</t>
+  </si>
+  <si>
+    <t>Severe;Mild</t>
+  </si>
+  <si>
+    <t>DOI: 10.1186/s13075-025-03489-9</t>
+  </si>
+  <si>
+    <t>TXT: PXD055158_experiment_annotation.txt</t>
+  </si>
+  <si>
+    <t>PXD045557</t>
+  </si>
+  <si>
+    <t>Lens</t>
+  </si>
+  <si>
+    <t>DC;ARC;PVC</t>
+  </si>
+  <si>
+    <t>DOI: 10.3390/jcm13237287</t>
+  </si>
+  <si>
+    <t>XLSX: PXD045557_KEY_Phaco.xlsx</t>
+  </si>
+  <si>
+    <t>PXD045554</t>
+  </si>
+  <si>
+    <t>Eye</t>
+  </si>
+  <si>
+    <t>XLSX: PXD045554_KEY_AH.xlsx</t>
+  </si>
+  <si>
+    <t>PXD054270</t>
+  </si>
+  <si>
+    <t>RWPE1/KSFM;RWPE1/MEMa;22Rv;LNCaP;PC3"</t>
+  </si>
+  <si>
+    <t>DOI: 10.3390/ANTIOX13111340</t>
+  </si>
+  <si>
+    <t>TXT: PXD054270_DIA_experimental_design_MCF001695.txt</t>
+  </si>
+  <si>
+    <t>PXD040451</t>
+  </si>
+  <si>
+    <t>Rectal cancer cell</t>
+  </si>
+  <si>
+    <t>Responder;Non-Responder</t>
+  </si>
+  <si>
+    <t>DOI: 10.3390/ijms242015412</t>
+  </si>
+  <si>
+    <t>XLSX: PXD040451_Key_30330.xlsx</t>
+  </si>
+  <si>
+    <t>PXD051606</t>
+  </si>
+  <si>
+    <t>Q Exactive HF-X;Orbitrap Exploris 480</t>
+  </si>
+  <si>
+    <t>Plasma</t>
+  </si>
+  <si>
+    <t>DOI: 10.1016/j.molmet.2024.101983</t>
+  </si>
+  <si>
+    <t>PXD043635</t>
+  </si>
+  <si>
+    <t>Veh;Dex;Spi10;Spi1;Dex+Spi10;Dex+Spi1</t>
+  </si>
+  <si>
+    <t>DOI: 10.1007/s00018-023-04900-x</t>
+  </si>
+  <si>
+    <t>TXT: PXD043635_sample_info.txt</t>
+  </si>
+  <si>
+    <t>PXD044220</t>
+  </si>
+  <si>
+    <t>Fibroblast</t>
+  </si>
+  <si>
+    <t>WT_D0;WT_D3;WT_D4;KO_D0;KO_D3;KO_D4</t>
+  </si>
+  <si>
+    <t>DOI: 10.3390/CANCERS15204997</t>
+  </si>
+  <si>
+    <t>XLSX: PXD044220_Dafou_KEY.xlsx</t>
+  </si>
+  <si>
+    <t>PXD054374</t>
+  </si>
+  <si>
+    <t>Vehicle;R1881</t>
+  </si>
+  <si>
+    <t>TXT: PXD054374_DIA_experimental_design_PCF000078.txt</t>
+  </si>
+  <si>
+    <t>PXD047024</t>
+  </si>
+  <si>
+    <t>Control;Mutant</t>
+  </si>
+  <si>
+    <t>XLSX: PXD047024_40485_KEY.xlsx</t>
+  </si>
+  <si>
+    <t>PXD047038</t>
+  </si>
+  <si>
+    <t>Es de Martina Samiotaki, xa teño moitos pero en ultima instancia valería</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>PXD054712</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do mesmo autor que PXD054636, pero valería </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> PXD051732</t>
+  </si>
+  <si>
+    <t>Do mesmo auto que PXD047566, valería</t>
+  </si>
+  <si>
+    <t>PXD041191</t>
+  </si>
+  <si>
+    <t>Es de Martina Samiotaki, pero é Sacaromyces…</t>
   </si>
 </sst>
 </file>
@@ -426,12 +886,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -758,9 +1219,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BCF4AC8-88B5-4543-8C52-FD30450BEA57}">
-  <dimension ref="A1:N51"/>
+  <dimension ref="A1:N61"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="2" max="2" width="13.28515625" customWidth="1"/>
     <col min="5" max="5" width="22.85546875" customWidth="1"/>
     <col min="6" max="6" width="15.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17.7109375" customWidth="1"/>
@@ -782,7 +1244,7 @@
         <v>1</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>2</v>
@@ -826,7 +1288,7 @@
         <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E2" t="s">
         <v>20</v>
@@ -871,7 +1333,7 @@
         <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E3" t="s">
         <v>20</v>
@@ -899,7 +1361,7 @@
         <v>29</v>
       </c>
       <c r="N3" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
@@ -913,7 +1375,7 @@
         <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E4" t="s">
         <v>12</v>
@@ -950,7 +1412,7 @@
         <v>8</v>
       </c>
       <c r="D5" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E5" t="s">
         <v>33</v>
@@ -989,7 +1451,7 @@
         <v>8</v>
       </c>
       <c r="D6" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E6" t="s">
         <v>38</v>
@@ -1019,7 +1481,7 @@
         <v>42</v>
       </c>
       <c r="N6" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
@@ -1033,7 +1495,7 @@
         <v>8</v>
       </c>
       <c r="D7" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E7" t="s">
         <v>45</v>
@@ -1064,7 +1526,7 @@
         <v>48</v>
       </c>
       <c r="N7" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
@@ -1078,7 +1540,7 @@
         <v>8</v>
       </c>
       <c r="D8" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E8" t="s">
         <v>50</v>
@@ -1121,7 +1583,7 @@
         <v>8</v>
       </c>
       <c r="D9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E9" t="s">
         <v>12</v>
@@ -1152,7 +1614,7 @@
         <v>54</v>
       </c>
       <c r="N9" t="s">
-        <v>60</v>
+        <v>105</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
@@ -1160,16 +1622,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" t="s">
+        <v>98</v>
+      </c>
+      <c r="E10" t="s">
         <v>61</v>
-      </c>
-      <c r="C10" t="s">
-        <v>8</v>
-      </c>
-      <c r="D10" t="s">
-        <v>100</v>
-      </c>
-      <c r="E10" t="s">
-        <v>62</v>
       </c>
       <c r="F10" t="s">
         <v>56</v>
@@ -1178,22 +1640,22 @@
         <v>11</v>
       </c>
       <c r="H10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I10">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J10" t="s">
-        <v>64</v>
+        <v>106</v>
       </c>
       <c r="K10">
         <v>24</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="N10" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
@@ -1201,16 +1663,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" t="s">
+        <v>98</v>
+      </c>
+      <c r="E11" t="s">
         <v>67</v>
-      </c>
-      <c r="C11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D11" t="s">
-        <v>100</v>
-      </c>
-      <c r="E11" t="s">
-        <v>69</v>
       </c>
       <c r="F11" t="s">
         <v>56</v>
@@ -1219,22 +1681,22 @@
         <v>11</v>
       </c>
       <c r="H11" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="I11">
         <v>2</v>
       </c>
       <c r="J11" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="K11">
         <v>33</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M11" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
@@ -1242,16 +1704,16 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C12" t="s">
         <v>8</v>
       </c>
       <c r="D12" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E12" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F12" t="s">
         <v>56</v>
@@ -1260,20 +1722,20 @@
         <v>18</v>
       </c>
       <c r="H12" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I12">
         <v>2</v>
       </c>
       <c r="J12" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="K12">
         <f>9</f>
         <v>9</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
@@ -1281,13 +1743,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C13" t="s">
         <v>8</v>
       </c>
       <c r="D13" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E13" t="s">
         <v>31</v>
@@ -1299,22 +1761,22 @@
         <v>18</v>
       </c>
       <c r="H13" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="I13">
         <v>2</v>
       </c>
       <c r="J13" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="K13">
         <v>16</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="N13" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
@@ -1322,13 +1784,13 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C14" t="s">
         <v>8</v>
       </c>
       <c r="D14" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E14" t="s">
         <v>50</v>
@@ -1340,23 +1802,23 @@
         <v>11</v>
       </c>
       <c r="H14" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="I14">
         <v>4</v>
       </c>
       <c r="J14" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="K14">
         <f>8*4</f>
         <v>32</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="N14" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
@@ -1364,16 +1826,16 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C15" t="s">
         <v>8</v>
       </c>
       <c r="D15" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F15" t="s">
         <v>9</v>
@@ -1382,251 +1844,1621 @@
         <v>11</v>
       </c>
       <c r="H15" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I15">
         <v>2</v>
       </c>
       <c r="J15" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="K15">
         <v>10</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="N15" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
+      <c r="B16" t="s">
+        <v>107</v>
+      </c>
+      <c r="C16" t="s">
+        <v>8</v>
+      </c>
       <c r="D16" t="s">
-        <v>100</v>
-      </c>
-      <c r="L16" s="1"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+        <v>98</v>
+      </c>
+      <c r="E16" t="s">
+        <v>108</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+      <c r="G16" t="s">
+        <v>11</v>
+      </c>
+      <c r="H16" t="s">
+        <v>77</v>
+      </c>
+      <c r="I16">
+        <v>3</v>
+      </c>
+      <c r="J16" t="s">
+        <v>109</v>
+      </c>
+      <c r="K16">
+        <v>9</v>
+      </c>
+      <c r="L16" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
+      <c r="B17" t="s">
+        <v>110</v>
+      </c>
+      <c r="C17" t="s">
+        <v>8</v>
+      </c>
       <c r="D17" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+        <v>98</v>
+      </c>
+      <c r="E17" t="s">
+        <v>31</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+      <c r="G17" t="s">
+        <v>11</v>
+      </c>
+      <c r="H17" t="s">
+        <v>111</v>
+      </c>
+      <c r="I17">
+        <v>2</v>
+      </c>
+      <c r="J17" t="s">
+        <v>112</v>
+      </c>
+      <c r="K17">
+        <v>46</v>
+      </c>
+      <c r="L17" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
+      <c r="B18" t="s">
+        <v>114</v>
+      </c>
+      <c r="C18" t="s">
+        <v>8</v>
+      </c>
       <c r="D18" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+        <v>98</v>
+      </c>
+      <c r="E18" t="s">
+        <v>71</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+      <c r="G18" t="s">
+        <v>11</v>
+      </c>
+      <c r="H18" t="s">
+        <v>115</v>
+      </c>
+      <c r="I18">
+        <v>2</v>
+      </c>
+      <c r="J18" t="s">
+        <v>116</v>
+      </c>
+      <c r="K18">
+        <v>6</v>
+      </c>
+      <c r="L18" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
+      <c r="B19" t="s">
+        <v>118</v>
+      </c>
+      <c r="C19" t="s">
+        <v>8</v>
+      </c>
       <c r="D19" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+        <v>98</v>
+      </c>
+      <c r="E19" t="s">
+        <v>31</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+      <c r="G19" t="s">
+        <v>11</v>
+      </c>
+      <c r="H19" t="s">
+        <v>39</v>
+      </c>
+      <c r="I19">
+        <v>3</v>
+      </c>
+      <c r="J19" t="s">
+        <v>119</v>
+      </c>
+      <c r="K19">
+        <f>I19*4</f>
+        <v>12</v>
+      </c>
+      <c r="L19" t="s">
+        <v>47</v>
+      </c>
+      <c r="N19" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
+      <c r="B20" t="s">
+        <v>121</v>
+      </c>
+      <c r="C20" t="s">
+        <v>8</v>
+      </c>
       <c r="D20" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+        <v>98</v>
+      </c>
+      <c r="E20" t="s">
+        <v>122</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+      <c r="G20" t="s">
+        <v>11</v>
+      </c>
+      <c r="H20" t="s">
+        <v>39</v>
+      </c>
+      <c r="I20">
+        <v>2</v>
+      </c>
+      <c r="J20" t="s">
+        <v>123</v>
+      </c>
+      <c r="K20">
+        <f>6</f>
+        <v>6</v>
+      </c>
+      <c r="L20" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="N20" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
+      <c r="B21" t="s">
+        <v>164</v>
+      </c>
+      <c r="C21" t="s">
+        <v>8</v>
+      </c>
       <c r="D21" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+        <v>98</v>
+      </c>
+      <c r="E21" t="s">
+        <v>33</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+      <c r="G21" t="s">
+        <v>160</v>
+      </c>
+      <c r="H21" t="s">
+        <v>39</v>
+      </c>
+      <c r="I21">
+        <v>8</v>
+      </c>
+      <c r="J21" t="s">
+        <v>166</v>
+      </c>
+      <c r="K21">
+        <f>I21*4</f>
+        <v>32</v>
+      </c>
+      <c r="L21" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="N21" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
+      <c r="B22" t="s">
+        <v>129</v>
+      </c>
+      <c r="C22" t="s">
+        <v>8</v>
+      </c>
       <c r="D22" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="E22" t="s">
+        <v>130</v>
+      </c>
+      <c r="F22" t="s">
+        <v>131</v>
+      </c>
+      <c r="G22" t="s">
+        <v>18</v>
+      </c>
+      <c r="H22" t="s">
+        <v>132</v>
+      </c>
+      <c r="I22">
+        <v>2</v>
+      </c>
+      <c r="J22" t="s">
+        <v>133</v>
+      </c>
+      <c r="K22">
+        <f>I22*11</f>
+        <v>22</v>
+      </c>
+      <c r="L22" t="s">
+        <v>47</v>
+      </c>
+      <c r="M22" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
+      <c r="B23" t="s">
+        <v>135</v>
+      </c>
+      <c r="C23" t="s">
+        <v>8</v>
+      </c>
       <c r="D23" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="E23" t="s">
+        <v>122</v>
+      </c>
+      <c r="F23" t="s">
+        <v>131</v>
+      </c>
+      <c r="G23" t="s">
+        <v>11</v>
+      </c>
+      <c r="H23" t="s">
+        <v>136</v>
+      </c>
+      <c r="I23">
+        <v>4</v>
+      </c>
+      <c r="J23" t="s">
+        <v>137</v>
+      </c>
+      <c r="K23">
+        <f>19*2+16*2+1</f>
+        <v>71</v>
+      </c>
+      <c r="L23" t="s">
+        <v>47</v>
+      </c>
+      <c r="N23" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
+      <c r="B24" t="s">
+        <v>139</v>
+      </c>
+      <c r="C24" t="s">
+        <v>8</v>
+      </c>
       <c r="D24" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="E24" t="s">
+        <v>122</v>
+      </c>
+      <c r="F24" t="s">
+        <v>131</v>
+      </c>
+      <c r="G24" t="s">
+        <v>11</v>
+      </c>
+      <c r="H24" t="s">
+        <v>115</v>
+      </c>
+      <c r="I24">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="J24" t="s">
+        <v>140</v>
+      </c>
+      <c r="K24">
+        <f>20</f>
+        <v>20</v>
+      </c>
+      <c r="L24" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
+      <c r="B25" t="s">
+        <v>142</v>
+      </c>
+      <c r="C25" t="s">
+        <v>8</v>
+      </c>
       <c r="D25" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="E25" t="s">
+        <v>143</v>
+      </c>
+      <c r="F25" t="s">
+        <v>131</v>
+      </c>
+      <c r="G25" t="s">
+        <v>11</v>
+      </c>
+      <c r="H25" t="s">
+        <v>144</v>
+      </c>
+      <c r="I25">
+        <v>3</v>
+      </c>
+      <c r="J25" t="s">
+        <v>145</v>
+      </c>
+      <c r="K25">
+        <v>46</v>
+      </c>
+      <c r="L25" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
+      <c r="B26" t="s">
+        <v>146</v>
+      </c>
+      <c r="C26" t="s">
+        <v>8</v>
+      </c>
       <c r="D26" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="E26" t="s">
+        <v>61</v>
+      </c>
+      <c r="F26" t="s">
+        <v>131</v>
+      </c>
+      <c r="G26" t="s">
+        <v>11</v>
+      </c>
+      <c r="H26" t="s">
+        <v>115</v>
+      </c>
+      <c r="I26">
+        <v>2</v>
+      </c>
+      <c r="J26" t="s">
+        <v>147</v>
+      </c>
+      <c r="K26">
+        <v>22</v>
+      </c>
+      <c r="L26" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
+      <c r="B27" t="s">
+        <v>148</v>
+      </c>
+      <c r="C27" t="s">
+        <v>8</v>
+      </c>
       <c r="D27" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="E27" t="s">
+        <v>45</v>
+      </c>
+      <c r="F27" t="s">
+        <v>131</v>
+      </c>
+      <c r="G27" t="s">
+        <v>18</v>
+      </c>
+      <c r="H27" t="s">
+        <v>39</v>
+      </c>
+      <c r="I27">
+        <v>5</v>
+      </c>
+      <c r="J27" t="s">
+        <v>149</v>
+      </c>
+      <c r="K27">
+        <f>I27*4</f>
+        <v>20</v>
+      </c>
+      <c r="L27" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
+      <c r="B28" t="s">
+        <v>150</v>
+      </c>
+      <c r="C28" t="s">
+        <v>8</v>
+      </c>
       <c r="D28" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="E28" t="s">
+        <v>45</v>
+      </c>
+      <c r="F28" t="s">
+        <v>131</v>
+      </c>
+      <c r="G28" t="s">
+        <v>18</v>
+      </c>
+      <c r="H28" t="s">
+        <v>132</v>
+      </c>
+      <c r="I28">
+        <v>3</v>
+      </c>
+      <c r="J28" t="s">
+        <v>151</v>
+      </c>
+      <c r="K28">
+        <f>I28*3</f>
+        <v>9</v>
+      </c>
+      <c r="L28" s="1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
+      <c r="B29" t="s">
+        <v>153</v>
+      </c>
+      <c r="C29" t="s">
+        <v>8</v>
+      </c>
       <c r="D29" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="E29" t="s">
+        <v>67</v>
+      </c>
+      <c r="F29" t="s">
+        <v>131</v>
+      </c>
+      <c r="G29" t="s">
+        <v>11</v>
+      </c>
+      <c r="H29" t="s">
+        <v>39</v>
+      </c>
+      <c r="I29">
+        <v>4</v>
+      </c>
+      <c r="J29" t="s">
+        <v>154</v>
+      </c>
+      <c r="K29">
+        <f>I29*3</f>
+        <v>12</v>
+      </c>
+      <c r="L29" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
+      <c r="B30" t="s">
+        <v>155</v>
+      </c>
+      <c r="C30" t="s">
+        <v>8</v>
+      </c>
       <c r="D30" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="E30" t="s">
+        <v>156</v>
+      </c>
+      <c r="F30" t="s">
+        <v>131</v>
+      </c>
+      <c r="G30" t="s">
+        <v>11</v>
+      </c>
+      <c r="H30" t="s">
+        <v>39</v>
+      </c>
+      <c r="I30">
+        <v>3</v>
+      </c>
+      <c r="J30" t="s">
+        <v>157</v>
+      </c>
+      <c r="K30">
+        <f>I30*4</f>
+        <v>12</v>
+      </c>
+      <c r="L30" s="1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
+      <c r="B31" t="s">
+        <v>159</v>
+      </c>
+      <c r="C31" t="s">
+        <v>8</v>
+      </c>
       <c r="D31" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="E31" t="s">
+        <v>161</v>
+      </c>
+      <c r="F31" t="s">
+        <v>131</v>
+      </c>
+      <c r="G31" t="s">
+        <v>160</v>
+      </c>
+      <c r="H31" t="s">
+        <v>39</v>
+      </c>
+      <c r="I31">
+        <v>4</v>
+      </c>
+      <c r="J31" t="s">
+        <v>162</v>
+      </c>
+      <c r="K31">
+        <f>I31*4</f>
+        <v>16</v>
+      </c>
+      <c r="L31" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B32" t="s">
+        <v>167</v>
+      </c>
+      <c r="C32" t="s">
+        <v>8</v>
+      </c>
+      <c r="D32" t="s">
+        <v>99</v>
+      </c>
+      <c r="E32" t="s">
+        <v>67</v>
+      </c>
+      <c r="F32" t="s">
+        <v>131</v>
+      </c>
+      <c r="G32" t="s">
+        <v>18</v>
+      </c>
+      <c r="H32" t="s">
+        <v>168</v>
+      </c>
+      <c r="I32">
+        <v>4</v>
+      </c>
+      <c r="J32" t="s">
+        <v>169</v>
+      </c>
+      <c r="K32">
+        <f>I32*4</f>
+        <v>16</v>
+      </c>
+      <c r="L32" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="M32" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B33" t="s">
+        <v>172</v>
+      </c>
+      <c r="C33" t="s">
+        <v>8</v>
+      </c>
+      <c r="D33" t="s">
+        <v>99</v>
+      </c>
+      <c r="E33" t="s">
+        <v>173</v>
+      </c>
+      <c r="F33" t="s">
+        <v>131</v>
+      </c>
+      <c r="G33" t="s">
+        <v>11</v>
+      </c>
+      <c r="H33" t="s">
+        <v>39</v>
+      </c>
+      <c r="I33">
+        <f>3</f>
+        <v>3</v>
+      </c>
+      <c r="J33" t="s">
+        <v>174</v>
+      </c>
+      <c r="K33">
+        <f>I33*3</f>
+        <v>9</v>
+      </c>
+      <c r="L33" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B34" t="s">
+        <v>176</v>
+      </c>
+      <c r="C34" t="s">
+        <v>8</v>
+      </c>
+      <c r="D34" t="s">
+        <v>99</v>
+      </c>
+      <c r="E34" t="s">
+        <v>31</v>
+      </c>
+      <c r="F34" t="s">
+        <v>131</v>
+      </c>
+      <c r="G34" t="s">
+        <v>18</v>
+      </c>
+      <c r="H34" t="s">
+        <v>177</v>
+      </c>
+      <c r="I34">
+        <v>4</v>
+      </c>
+      <c r="J34" t="s">
+        <v>178</v>
+      </c>
+      <c r="K34">
+        <f>11</f>
+        <v>11</v>
+      </c>
+      <c r="L34" s="1" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B35" t="s">
+        <v>180</v>
+      </c>
+      <c r="C35" t="s">
+        <v>8</v>
+      </c>
+      <c r="D35" t="s">
+        <v>99</v>
+      </c>
+      <c r="E35" t="s">
+        <v>12</v>
+      </c>
+      <c r="F35" t="s">
+        <v>131</v>
+      </c>
+      <c r="G35" t="s">
+        <v>11</v>
+      </c>
+      <c r="H35" t="s">
+        <v>181</v>
+      </c>
+      <c r="I35">
+        <v>3</v>
+      </c>
+      <c r="J35" t="s">
+        <v>182</v>
+      </c>
+      <c r="K35">
+        <f>9</f>
+        <v>9</v>
+      </c>
+      <c r="L35" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B36" t="s">
+        <v>183</v>
+      </c>
+      <c r="C36" t="s">
+        <v>8</v>
+      </c>
+      <c r="D36" t="s">
+        <v>99</v>
+      </c>
+      <c r="E36" t="s">
+        <v>187</v>
+      </c>
+      <c r="F36" t="s">
+        <v>131</v>
+      </c>
+      <c r="G36" t="s">
+        <v>11</v>
+      </c>
+      <c r="H36" t="s">
+        <v>186</v>
+      </c>
+      <c r="I36">
+        <v>2</v>
+      </c>
+      <c r="J36" t="s">
+        <v>184</v>
+      </c>
+      <c r="K36">
+        <f>8</f>
+        <v>8</v>
+      </c>
+      <c r="L36" s="1" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B37" t="s">
+        <v>188</v>
+      </c>
+      <c r="C37" t="s">
+        <v>8</v>
+      </c>
+      <c r="D37" t="s">
+        <v>99</v>
+      </c>
+      <c r="E37" t="s">
+        <v>71</v>
+      </c>
+      <c r="F37" t="s">
+        <v>131</v>
+      </c>
+      <c r="G37" t="s">
+        <v>11</v>
+      </c>
+      <c r="H37" t="s">
+        <v>136</v>
+      </c>
+      <c r="I37">
+        <v>2</v>
+      </c>
+      <c r="J37" t="s">
+        <v>189</v>
+      </c>
+      <c r="K37">
+        <f>25*2</f>
+        <v>50</v>
+      </c>
+      <c r="L37" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="M37" t="s">
+        <v>190</v>
+      </c>
+      <c r="N37" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B38" t="s">
+        <v>193</v>
+      </c>
+      <c r="C38" t="s">
+        <v>8</v>
+      </c>
+      <c r="D38" t="s">
+        <v>99</v>
+      </c>
+      <c r="E38" t="s">
+        <v>31</v>
+      </c>
+      <c r="F38" t="s">
+        <v>131</v>
+      </c>
+      <c r="G38" t="s">
+        <v>18</v>
+      </c>
+      <c r="H38" t="s">
+        <v>39</v>
+      </c>
+      <c r="I38">
+        <v>2</v>
+      </c>
+      <c r="J38" t="s">
+        <v>194</v>
+      </c>
+      <c r="K38">
+        <f>6</f>
+        <v>6</v>
+      </c>
+      <c r="L38" s="1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B39" t="s">
+        <v>196</v>
+      </c>
+      <c r="C39" t="s">
+        <v>8</v>
+      </c>
+      <c r="D39" t="s">
+        <v>99</v>
+      </c>
+      <c r="E39" t="s">
+        <v>197</v>
+      </c>
+      <c r="F39" t="s">
+        <v>131</v>
+      </c>
+      <c r="G39" t="s">
+        <v>11</v>
+      </c>
+      <c r="H39" t="s">
+        <v>198</v>
+      </c>
+      <c r="I39">
+        <v>4</v>
+      </c>
+      <c r="J39" t="s">
+        <v>199</v>
+      </c>
+      <c r="K39">
+        <f>I39*3</f>
+        <v>12</v>
+      </c>
+      <c r="L39" s="1" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B40" t="s">
+        <v>201</v>
+      </c>
+      <c r="C40" t="s">
+        <v>8</v>
+      </c>
+      <c r="D40" t="s">
+        <v>99</v>
+      </c>
+      <c r="E40" t="s">
+        <v>61</v>
+      </c>
+      <c r="F40" t="s">
+        <v>131</v>
+      </c>
+      <c r="G40" t="s">
+        <v>11</v>
+      </c>
+      <c r="H40" t="s">
+        <v>144</v>
+      </c>
+      <c r="I40">
+        <v>4</v>
+      </c>
+      <c r="J40" t="s">
+        <v>202</v>
+      </c>
+      <c r="K40">
+        <f>I40*10</f>
+        <v>40</v>
+      </c>
+      <c r="L40" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="M40" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B41" t="s">
+        <v>205</v>
+      </c>
+      <c r="C41" t="s">
+        <v>8</v>
+      </c>
+      <c r="D41" t="s">
+        <v>99</v>
+      </c>
+      <c r="E41" t="s">
+        <v>67</v>
+      </c>
+      <c r="F41" t="s">
+        <v>131</v>
+      </c>
+      <c r="G41" t="s">
+        <v>18</v>
+      </c>
+      <c r="H41" t="s">
+        <v>77</v>
+      </c>
+      <c r="I41">
+        <v>4</v>
+      </c>
+      <c r="J41" t="s">
+        <v>206</v>
+      </c>
+      <c r="K41">
+        <f>24</f>
+        <v>24</v>
+      </c>
+      <c r="L41" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="M41" t="s">
+        <v>208</v>
+      </c>
+      <c r="N41" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B42" t="s">
+        <v>128</v>
+      </c>
+      <c r="C42" t="s">
+        <v>8</v>
+      </c>
+      <c r="D42" t="s">
+        <v>98</v>
+      </c>
+      <c r="E42" t="s">
+        <v>122</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+      <c r="G42" t="s">
+        <v>11</v>
+      </c>
+      <c r="H42" t="s">
+        <v>39</v>
+      </c>
+      <c r="I42">
+        <v>2</v>
+      </c>
+      <c r="J42" t="s">
+        <v>127</v>
+      </c>
+      <c r="K42">
+        <f>6</f>
+        <v>6</v>
+      </c>
+      <c r="L42" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="N42" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B43" t="s">
+        <v>210</v>
+      </c>
+      <c r="C43" t="s">
+        <v>8</v>
+      </c>
+      <c r="D43" t="s">
+        <v>99</v>
+      </c>
+      <c r="E43" t="s">
+        <v>211</v>
+      </c>
+      <c r="F43" t="s">
+        <v>131</v>
+      </c>
+      <c r="G43" t="s">
+        <v>11</v>
+      </c>
+      <c r="H43" t="s">
+        <v>115</v>
+      </c>
+      <c r="I43">
+        <v>2</v>
+      </c>
+      <c r="J43" t="s">
+        <v>212</v>
+      </c>
+      <c r="K43">
+        <f>35</f>
+        <v>35</v>
+      </c>
+      <c r="L43" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="M43" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B44" t="s">
+        <v>215</v>
+      </c>
+      <c r="C44" t="s">
+        <v>8</v>
+      </c>
+      <c r="D44" t="s">
+        <v>99</v>
+      </c>
+      <c r="E44" t="s">
+        <v>20</v>
+      </c>
+      <c r="F44" t="s">
+        <v>131</v>
+      </c>
+      <c r="G44" t="s">
+        <v>11</v>
+      </c>
+      <c r="H44" t="s">
+        <v>216</v>
+      </c>
+      <c r="I44">
+        <v>3</v>
+      </c>
+      <c r="J44" t="s">
+        <v>217</v>
+      </c>
+      <c r="K44">
+        <v>29</v>
+      </c>
+      <c r="L44" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="M44" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B45" t="s">
+        <v>220</v>
+      </c>
+      <c r="C45" t="s">
+        <v>8</v>
+      </c>
+      <c r="D45" t="s">
+        <v>99</v>
+      </c>
+      <c r="E45" t="s">
+        <v>20</v>
+      </c>
+      <c r="F45" t="s">
+        <v>131</v>
+      </c>
+      <c r="G45" t="s">
+        <v>11</v>
+      </c>
+      <c r="H45" t="s">
+        <v>221</v>
+      </c>
+      <c r="I45">
+        <v>3</v>
+      </c>
+      <c r="J45" t="s">
+        <v>217</v>
+      </c>
+      <c r="K45">
+        <v>28</v>
+      </c>
+      <c r="L45" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="M45" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B46" t="s">
+        <v>223</v>
+      </c>
+      <c r="C46" t="s">
+        <v>8</v>
+      </c>
+      <c r="D46" t="s">
+        <v>99</v>
+      </c>
+      <c r="E46" t="s">
+        <v>130</v>
+      </c>
+      <c r="F46" t="s">
+        <v>131</v>
+      </c>
+      <c r="G46" t="s">
+        <v>11</v>
+      </c>
+      <c r="H46" t="s">
+        <v>39</v>
+      </c>
+      <c r="I46">
+        <v>6</v>
+      </c>
+      <c r="J46" t="s">
+        <v>224</v>
+      </c>
+      <c r="K46">
+        <f>6*3</f>
+        <v>18</v>
+      </c>
+      <c r="L46" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="M46" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B47" t="s">
+        <v>227</v>
+      </c>
+      <c r="C47" t="s">
+        <v>8</v>
+      </c>
+      <c r="D47" t="s">
+        <v>99</v>
+      </c>
+      <c r="E47" t="s">
+        <v>20</v>
+      </c>
+      <c r="F47" t="s">
+        <v>131</v>
+      </c>
+      <c r="G47" t="s">
+        <v>11</v>
+      </c>
+      <c r="H47" t="s">
+        <v>228</v>
+      </c>
+      <c r="I47">
+        <v>2</v>
+      </c>
+      <c r="J47" t="s">
+        <v>229</v>
+      </c>
+      <c r="K47">
+        <v>21</v>
+      </c>
+      <c r="L47" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="M47" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B48" t="s">
+        <v>232</v>
+      </c>
+      <c r="C48" t="s">
+        <v>8</v>
+      </c>
+      <c r="D48" t="s">
+        <v>99</v>
+      </c>
+      <c r="E48" t="s">
+        <v>233</v>
+      </c>
+      <c r="F48" t="s">
+        <v>131</v>
+      </c>
+      <c r="G48" t="s">
+        <v>18</v>
+      </c>
+      <c r="H48" t="s">
+        <v>234</v>
+      </c>
+      <c r="I48">
+        <v>2</v>
+      </c>
+      <c r="J48" t="s">
+        <v>74</v>
+      </c>
+      <c r="K48">
+        <v>8</v>
+      </c>
+      <c r="L48" s="1" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B49" t="s">
+        <v>236</v>
+      </c>
+      <c r="C49" t="s">
+        <v>8</v>
+      </c>
+      <c r="D49" t="s">
+        <v>99</v>
+      </c>
+      <c r="E49" t="s">
+        <v>45</v>
+      </c>
+      <c r="F49" t="s">
+        <v>131</v>
+      </c>
+      <c r="G49" t="s">
+        <v>11</v>
+      </c>
+      <c r="H49" t="s">
+        <v>39</v>
+      </c>
+      <c r="I49">
+        <v>6</v>
+      </c>
+      <c r="J49" t="s">
+        <v>237</v>
+      </c>
+      <c r="K49">
+        <f>I49*4</f>
+        <v>24</v>
+      </c>
+      <c r="L49" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="M49" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B50" t="s">
+        <v>240</v>
+      </c>
+      <c r="C50" t="s">
+        <v>8</v>
+      </c>
+      <c r="D50" t="s">
+        <v>99</v>
+      </c>
+      <c r="E50" t="s">
+        <v>20</v>
+      </c>
+      <c r="F50" t="s">
+        <v>131</v>
+      </c>
+      <c r="G50" t="s">
+        <v>18</v>
+      </c>
+      <c r="H50" t="s">
+        <v>241</v>
+      </c>
+      <c r="I50">
+        <f>6</f>
+        <v>6</v>
+      </c>
+      <c r="J50" t="s">
+        <v>242</v>
+      </c>
+      <c r="K50">
+        <f>I50*3</f>
+        <v>18</v>
+      </c>
+      <c r="L50" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="M50" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
+      </c>
+      <c r="B51" t="s">
+        <v>245</v>
+      </c>
+      <c r="C51" t="s">
+        <v>8</v>
+      </c>
+      <c r="D51" t="s">
+        <v>99</v>
+      </c>
+      <c r="E51" t="s">
+        <v>130</v>
+      </c>
+      <c r="F51" t="s">
+        <v>131</v>
+      </c>
+      <c r="G51" t="s">
+        <v>11</v>
+      </c>
+      <c r="H51" t="s">
+        <v>39</v>
+      </c>
+      <c r="I51">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="J51" t="s">
+        <v>246</v>
+      </c>
+      <c r="K51">
+        <f>I51*3</f>
+        <v>6</v>
+      </c>
+      <c r="L51" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="M51" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="s">
+        <v>248</v>
+      </c>
+      <c r="C52" t="s">
+        <v>8</v>
+      </c>
+      <c r="D52" t="s">
+        <v>99</v>
+      </c>
+      <c r="E52" t="s">
+        <v>20</v>
+      </c>
+      <c r="F52" t="s">
+        <v>131</v>
+      </c>
+      <c r="G52" t="s">
+        <v>18</v>
+      </c>
+      <c r="H52" t="s">
+        <v>241</v>
+      </c>
+      <c r="I52">
+        <v>2</v>
+      </c>
+      <c r="J52" t="s">
+        <v>249</v>
+      </c>
+      <c r="K52">
+        <v>6</v>
+      </c>
+      <c r="L52" t="s">
+        <v>47</v>
+      </c>
+      <c r="M52" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="C53" t="s">
+        <v>8</v>
+      </c>
+      <c r="D53" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="C54" t="s">
+        <v>8</v>
+      </c>
+      <c r="D54" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="C55" t="s">
+        <v>8</v>
+      </c>
+      <c r="D55" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="C56" t="s">
+        <v>8</v>
+      </c>
+      <c r="D56" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="C57" t="s">
+        <v>8</v>
+      </c>
+      <c r="D57" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="C58" t="s">
+        <v>8</v>
+      </c>
+      <c r="D58" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="C59" t="s">
+        <v>8</v>
+      </c>
+      <c r="D59" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="C60" t="s">
+        <v>8</v>
+      </c>
+      <c r="D60" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="C61" t="s">
+        <v>8</v>
+      </c>
+      <c r="D61" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1644,9 +3476,36 @@
     <hyperlink ref="L13" r:id="rId11" location="Sec11" xr:uid="{EAAEE3D5-FD5F-4C5E-BEDE-E149007B61D7}"/>
     <hyperlink ref="L14" r:id="rId12" xr:uid="{1466ACE4-040B-4872-B3E7-CB073BC90CE4}"/>
     <hyperlink ref="L15" r:id="rId13" display="https://doi.org/10.1038/s42255-021-00420-9" xr:uid="{AA76EE2A-3D95-4B26-A3B2-D6961FCAA8B9}"/>
+    <hyperlink ref="L17" r:id="rId14" xr:uid="{73C3C164-1B9E-424D-B497-0A5C1413062E}"/>
+    <hyperlink ref="L18" r:id="rId15" xr:uid="{8E96941A-F27E-446D-BAAB-8817BA69407F}"/>
+    <hyperlink ref="L20" r:id="rId16" xr:uid="{612CAC31-BDF9-4217-882E-04BA9D317851}"/>
+    <hyperlink ref="L42" r:id="rId17" xr:uid="{A0AABACF-D49B-4ADE-969F-34674947E980}"/>
+    <hyperlink ref="L24" r:id="rId18" xr:uid="{45029A78-EC32-4653-B2C0-8A1C6AB739CD}"/>
+    <hyperlink ref="L28" r:id="rId19" xr:uid="{58E39B3E-0FD0-41D5-8918-94CB0DEBE92F}"/>
+    <hyperlink ref="L30" r:id="rId20" xr:uid="{798BD1EC-17B3-4197-8EAE-486722AEADF1}"/>
+    <hyperlink ref="L31" r:id="rId21" xr:uid="{AE40AA44-2798-47B6-B9FB-02DFCD819A98}"/>
+    <hyperlink ref="L21" r:id="rId22" xr:uid="{812AD498-467D-4930-99B1-0BD72991EB74}"/>
+    <hyperlink ref="L32" r:id="rId23" xr:uid="{0A4265F2-3C05-4E25-883C-F8A8F58C6D63}"/>
+    <hyperlink ref="L33" r:id="rId24" xr:uid="{DBE6CDEE-1512-471E-91A3-29DE9DCD40F4}"/>
+    <hyperlink ref="L34" r:id="rId25" xr:uid="{1530F3E7-5FB8-4C45-8815-BC53BEE62E5F}"/>
+    <hyperlink ref="L36" r:id="rId26" xr:uid="{81A03F1A-4A0B-4C2D-947D-86D4D18A30FC}"/>
+    <hyperlink ref="L37" r:id="rId27" xr:uid="{03A7BDDE-DDD3-4CE4-9A6A-3F28026978CD}"/>
+    <hyperlink ref="L38" r:id="rId28" xr:uid="{97D5A0D0-4F73-4447-98D7-176FE36E7E9F}"/>
+    <hyperlink ref="L39" r:id="rId29" xr:uid="{3FDDCA56-CB99-4846-8D3C-3F87979E1526}"/>
+    <hyperlink ref="L40" r:id="rId30" xr:uid="{7859E8C3-2333-43D3-B478-A44FA49BB177}"/>
+    <hyperlink ref="L41" r:id="rId31" xr:uid="{4AAB6572-69BF-4A8C-B9DD-0ECD744015A7}"/>
+    <hyperlink ref="L43" r:id="rId32" xr:uid="{AEFB8F3B-EA1A-47CE-B2E9-52C8FEE30E73}"/>
+    <hyperlink ref="L44" r:id="rId33" xr:uid="{CB2F7DF2-FC97-4B92-86B1-9479DA20F40F}"/>
+    <hyperlink ref="L45" r:id="rId34" xr:uid="{256ADA76-DDF3-43D7-9FF6-3D06B3102F1B}"/>
+    <hyperlink ref="L46" r:id="rId35" xr:uid="{8607D0FC-A3CA-4C2C-B9AF-EA3A5742473F}"/>
+    <hyperlink ref="L47" r:id="rId36" xr:uid="{CC518961-8295-4994-A3DF-84ED80F14808}"/>
+    <hyperlink ref="L48" r:id="rId37" xr:uid="{2FCAA5AF-4D5B-40D6-9710-958A63043040}"/>
+    <hyperlink ref="L49" r:id="rId38" xr:uid="{AE407C0D-97C6-498B-BFB4-71C4936A1365}"/>
+    <hyperlink ref="L50" r:id="rId39" xr:uid="{92FB0A8D-11DB-4567-8F9B-CF523A119E05}"/>
+    <hyperlink ref="L51" r:id="rId40" xr:uid="{207EE6F5-656D-4A38-9817-F2A00ABFCEEE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId14"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId41"/>
 </worksheet>
 </file>
 
@@ -1666,10 +3525,10 @@
         <v>1</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>2</v>
@@ -1707,46 +3566,46 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F2" t="s">
         <v>31</v>
       </c>
       <c r="G2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="H2" t="s">
         <v>11</v>
       </c>
       <c r="I2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="J2">
         <v>7</v>
       </c>
       <c r="K2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="L2">
         <v>365</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="N2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="O2" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -1755,4 +3614,57 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5412E459-6599-4D39-A6E4-9FCCBAA2B3FA}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="65.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>251</v>
+      </c>
+      <c r="B2" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>254</v>
+      </c>
+      <c r="B3" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>256</v>
+      </c>
+      <c r="B4" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>258</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>259</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Database of gold standard datasets completed!
</commit_message>
<xml_diff>
--- a/goldStandard/_Index.xlsx
+++ b/goldStandard/_Index.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julia\Documents\GitHub\normScore\goldStandard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9342C580-29F6-45ED-917A-31FFFF31A0C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE5062FE-6E5A-460F-8B06-332CF3AFEA76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24960" yWindow="0" windowWidth="26745" windowHeight="20985" xr2:uid="{F827C457-048B-4104-BF2A-59E43A6422D6}"/>
+    <workbookView xWindow="-19320" yWindow="-2745" windowWidth="19440" windowHeight="14880" xr2:uid="{F827C457-048B-4104-BF2A-59E43A6422D6}"/>
   </bookViews>
   <sheets>
     <sheet name="In" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="892" uniqueCount="399">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1028" uniqueCount="476">
   <si>
     <t>ID</t>
   </si>
@@ -1199,9 +1199,6 @@
     <t>DOI: 10.3390/antiox12061153</t>
   </si>
   <si>
-    <t>https://www.ebi.ac.uk/pride/archive?keyword=proteinGroups.txt&amp;filter=projectTags%3D%3DBiology%2Fdisease-driven%20human%20proteome%20project%20%28b%2Fd-hpp%29&amp;sortFields=downloadCount&amp;sortDirection=DESC&amp;page=0&amp;pageSize=20</t>
-  </si>
-  <si>
     <t>PXD040288</t>
   </si>
   <si>
@@ -1227,6 +1224,240 @@
   </si>
   <si>
     <t>Ctrl;XAV939</t>
+  </si>
+  <si>
+    <t>PXD042498</t>
+  </si>
+  <si>
+    <t>DMSO_24hr;DMSO_4hr;ERCO_24hr;ERCO_4hr</t>
+  </si>
+  <si>
+    <t>DOI: 10.12688/openreseurope.15973.2</t>
+  </si>
+  <si>
+    <t>Hsp162_Insolubl;Hsp162_Solubl;Hsp17_Insolubl;Hsp17_Solubl;Insolubl;Sip1_Insolubl;Sip1_Solubl;Solubl</t>
+  </si>
+  <si>
+    <t>PXD038019</t>
+  </si>
+  <si>
+    <t>DOI: 10.1016/J.JBC.2022.102753</t>
+  </si>
+  <si>
+    <t>PXD069093</t>
+  </si>
+  <si>
+    <t>XLSX: PXD069093_KinomeMetadata.xlsx</t>
+  </si>
+  <si>
+    <t>palbociclib;palbociclib_efficacy;vehicle;vehicle_efficacy</t>
+  </si>
+  <si>
+    <t>Xenografs</t>
+  </si>
+  <si>
+    <t>DOI: 10.1016/j.neo.2025.101266</t>
+  </si>
+  <si>
+    <t>PXD068908</t>
+  </si>
+  <si>
+    <t>3T3L1_Co;3T3L1_Vas;imBA_Co;imBA_Vas</t>
+  </si>
+  <si>
+    <t>DOI: 10.1038/s41467-025-66950-y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bad quality, many missing values and two types of cell cultures that should be independently analyzed </t>
+  </si>
+  <si>
+    <t>PXD068664</t>
+  </si>
+  <si>
+    <t>Cell culture, 3x3 samples</t>
+  </si>
+  <si>
+    <t>PXD004242</t>
+  </si>
+  <si>
+    <t>Only one group: obesity</t>
+  </si>
+  <si>
+    <t>PXD005354</t>
+  </si>
+  <si>
+    <t>Only one group: colorrectal cancer</t>
+  </si>
+  <si>
+    <t>PXD005025</t>
+  </si>
+  <si>
+    <t>Vigna mungo</t>
+  </si>
+  <si>
+    <t>Leaves</t>
+  </si>
+  <si>
+    <t>V2;SV2;V6;SV6;S6;C2;C6;S2</t>
+  </si>
+  <si>
+    <t>DOI: 10.1021/acs.jproteome.6b00211</t>
+  </si>
+  <si>
+    <t>PXD027404</t>
+  </si>
+  <si>
+    <t>Only one group: Adenocarcinoma</t>
+  </si>
+  <si>
+    <t>PXD010785</t>
+  </si>
+  <si>
+    <t>DMSO;xanthohumol C in DMSO;xanthohumol in DMSO</t>
+  </si>
+  <si>
+    <t>DOI: 10.1371/journal.pone.0213469</t>
+  </si>
+  <si>
+    <t>PXD022701</t>
+  </si>
+  <si>
+    <t>Drosophila melanogaster</t>
+  </si>
+  <si>
+    <t>Head</t>
+  </si>
+  <si>
+    <t>C;E</t>
+  </si>
+  <si>
+    <t>DOI: 10.1016/j.jbc.2021.100408</t>
+  </si>
+  <si>
+    <t>HTLV1a;HTLV1c;Mock</t>
+  </si>
+  <si>
+    <t>T-cell</t>
+  </si>
+  <si>
+    <t> PXD030132</t>
+  </si>
+  <si>
+    <t>DOI: 10.1016/J.CELL.2025.06.023</t>
+  </si>
+  <si>
+    <t>PXD028841</t>
+  </si>
+  <si>
+    <t>BD;CON;FEP;MDD</t>
+  </si>
+  <si>
+    <t>DOI: 10.1016/j.dib.2021.107495</t>
+  </si>
+  <si>
+    <t>PXD015470</t>
+  </si>
+  <si>
+    <t>Ovary</t>
+  </si>
+  <si>
+    <t>AA;C</t>
+  </si>
+  <si>
+    <t>DOI: 10.1007/s00204-020-02697-3</t>
+  </si>
+  <si>
+    <t>PXD020238</t>
+  </si>
+  <si>
+    <t>Sodium butyrate;Untreated</t>
+  </si>
+  <si>
+    <t>Canis familiaris</t>
+  </si>
+  <si>
+    <t>PXD020245</t>
+  </si>
+  <si>
+    <t>Untreated_Ileum;Untreated_Distal Colon;Untreated_Proximal Colon;Treated_Ileum;Treated_Distal Colon;Treated_Proximal Colon</t>
+  </si>
+  <si>
+    <t>Intestin</t>
+  </si>
+  <si>
+    <t>DOI: 10.1016/j.xphs.2020.11.001</t>
+  </si>
+  <si>
+    <t>PXD062946</t>
+  </si>
+  <si>
+    <t>Crtl_antiFLAG;Crtl_antiGFP;hangover_FLAG;hangover_GFP</t>
+  </si>
+  <si>
+    <t>PXD011804</t>
+  </si>
+  <si>
+    <t>CAA;N;PDF</t>
+  </si>
+  <si>
+    <t>DOI: 10.1021/acs.jproteome.9b00242</t>
+  </si>
+  <si>
+    <t>DOI: 10.1093/nar/gkaf1349</t>
+  </si>
+  <si>
+    <t>Nash;Norm;SS</t>
+  </si>
+  <si>
+    <t>PXD005847</t>
+  </si>
+  <si>
+    <t>LTQ Orbitrap Velos</t>
+  </si>
+  <si>
+    <t>DOI: 10.1186/s12014-018-9186-0</t>
+  </si>
+  <si>
+    <t>Case;Wild Control;Captive Control</t>
+  </si>
+  <si>
+    <t>PXD030595</t>
+  </si>
+  <si>
+    <t>Enhydra lutris nereis</t>
+  </si>
+  <si>
+    <t>APP;KYL;WT</t>
+  </si>
+  <si>
+    <t>PXD056771</t>
+  </si>
+  <si>
+    <t>DOI: 10.1073/PNAS.2420324122</t>
+  </si>
+  <si>
+    <t>XLSX: PXD030595_Table_S1.xlsx</t>
+  </si>
+  <si>
+    <t>TXT: PXD005847_experimentalDesignTemplate.txt</t>
+  </si>
+  <si>
+    <t>TXT: PXD062946_experimentalDesignTemplate.txt</t>
+  </si>
+  <si>
+    <t>TXT: PXD020245_metadata_Mouse.txt</t>
+  </si>
+  <si>
+    <t>TXT: PXD020238_metadata_NaBut.txt</t>
+  </si>
+  <si>
+    <t>XLSX: PXD015470_metadata.xlsx</t>
+  </si>
+  <si>
+    <t>TXT: PXD005025_experimentalDesignTemplate.txt</t>
+  </si>
+  <si>
+    <t>PXD022038_Conditionsassessed.xlsx</t>
   </si>
 </sst>
 </file>
@@ -1306,12 +1537,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -1639,20 +1871,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BCF4AC8-88B5-4543-8C52-FD30450BEA57}">
   <dimension ref="A1:N102"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="13.28515625" customWidth="1"/>
-    <col min="5" max="5" width="22.85546875" customWidth="1"/>
-    <col min="6" max="6" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.7109375" customWidth="1"/>
-    <col min="8" max="8" width="27.85546875" customWidth="1"/>
-    <col min="10" max="10" width="14.28515625" customWidth="1"/>
-    <col min="12" max="12" width="38.28515625" customWidth="1"/>
-    <col min="13" max="13" width="40.7109375" customWidth="1"/>
-    <col min="14" max="14" width="38.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.3046875" customWidth="1"/>
+    <col min="5" max="5" width="22.84375" customWidth="1"/>
+    <col min="6" max="6" width="15.3046875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.69140625" customWidth="1"/>
+    <col min="8" max="8" width="27.84375" customWidth="1"/>
+    <col min="10" max="10" width="14.3046875" customWidth="1"/>
+    <col min="12" max="12" width="38.3046875" customWidth="1"/>
+    <col min="13" max="13" width="40.69140625" customWidth="1"/>
+    <col min="14" max="14" width="38.3828125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" s="2" customFormat="1" ht="15.9" x14ac:dyDescent="0.45">
       <c r="A1" s="2" t="s">
         <v>43</v>
       </c>
@@ -1696,7 +1928,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1741,7 +1973,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1783,7 +2015,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1820,7 +2052,7 @@
       </c>
       <c r="M4" s="1"/>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1859,7 +2091,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1903,7 +2135,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1948,7 +2180,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1991,7 +2223,7 @@
       </c>
       <c r="N8" s="4"/>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2036,7 +2268,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2077,7 +2309,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2118,7 +2350,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2157,7 +2389,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2198,7 +2430,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2240,7 +2472,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2281,7 +2513,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2319,7 +2551,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A17">
         <v>16</v>
       </c>
@@ -2357,7 +2589,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A18">
         <v>17</v>
       </c>
@@ -2395,7 +2627,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2437,7 +2669,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A20">
         <v>19</v>
       </c>
@@ -2478,7 +2710,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A21">
         <v>20</v>
       </c>
@@ -2520,7 +2752,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A22">
         <v>21</v>
       </c>
@@ -2562,7 +2794,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A23">
         <v>22</v>
       </c>
@@ -2604,7 +2836,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A24">
         <v>23</v>
       </c>
@@ -2644,7 +2876,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A25">
         <v>24</v>
       </c>
@@ -2682,7 +2914,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A26">
         <v>25</v>
       </c>
@@ -2720,7 +2952,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A27">
         <v>26</v>
       </c>
@@ -2759,7 +2991,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2798,7 +3030,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A29">
         <v>28</v>
       </c>
@@ -2837,7 +3069,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A30">
         <v>29</v>
       </c>
@@ -2876,7 +3108,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A31">
         <v>30</v>
       </c>
@@ -2915,7 +3147,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A32">
         <v>31</v>
       </c>
@@ -2957,7 +3189,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A33">
         <v>32</v>
       </c>
@@ -2997,7 +3229,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A34">
         <v>33</v>
       </c>
@@ -3036,7 +3268,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A35">
         <v>34</v>
       </c>
@@ -3075,7 +3307,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A36">
         <v>35</v>
       </c>
@@ -3114,7 +3346,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A37">
         <v>36</v>
       </c>
@@ -3159,7 +3391,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A38">
         <v>37</v>
       </c>
@@ -3198,7 +3430,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A39">
         <v>38</v>
       </c>
@@ -3237,7 +3469,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A40">
         <v>39</v>
       </c>
@@ -3279,7 +3511,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A41">
         <v>40</v>
       </c>
@@ -3324,7 +3556,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A42">
         <v>41</v>
       </c>
@@ -3366,7 +3598,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A43">
         <v>42</v>
       </c>
@@ -3408,7 +3640,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A44">
         <v>43</v>
       </c>
@@ -3449,7 +3681,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A45">
         <v>44</v>
       </c>
@@ -3490,7 +3722,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A46">
         <v>45</v>
       </c>
@@ -3532,7 +3764,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A47">
         <v>46</v>
       </c>
@@ -3573,7 +3805,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A48">
         <v>47</v>
       </c>
@@ -3611,7 +3843,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A49">
         <v>48</v>
       </c>
@@ -3653,7 +3885,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A50">
         <v>49</v>
       </c>
@@ -3696,7 +3928,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A51">
         <v>50</v>
       </c>
@@ -3739,7 +3971,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A52">
         <v>51</v>
       </c>
@@ -3780,7 +4012,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A53">
         <v>52</v>
       </c>
@@ -3824,7 +4056,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A54">
         <v>53</v>
       </c>
@@ -3866,7 +4098,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A55">
         <v>54</v>
       </c>
@@ -3908,7 +4140,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A56">
         <v>55</v>
       </c>
@@ -3950,7 +4182,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A57">
         <v>56</v>
       </c>
@@ -3992,7 +4224,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A58">
         <v>57</v>
       </c>
@@ -4033,7 +4265,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A59">
         <v>58</v>
       </c>
@@ -4074,7 +4306,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A60">
         <v>59</v>
       </c>
@@ -4115,7 +4347,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A61">
         <v>60</v>
       </c>
@@ -4160,7 +4392,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A62">
         <v>61</v>
       </c>
@@ -4202,7 +4434,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A63">
         <v>62</v>
       </c>
@@ -4243,7 +4475,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A64">
         <v>63</v>
       </c>
@@ -4284,7 +4516,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A65">
         <v>64</v>
       </c>
@@ -4325,7 +4557,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A66">
         <v>65</v>
       </c>
@@ -4364,7 +4596,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A67">
         <v>66</v>
       </c>
@@ -4406,7 +4638,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A68">
         <v>67</v>
       </c>
@@ -4444,7 +4676,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A69">
         <v>68</v>
       </c>
@@ -4483,7 +4715,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A70">
         <v>69</v>
       </c>
@@ -4524,7 +4756,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A71">
         <v>70</v>
       </c>
@@ -4566,7 +4798,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A72">
         <v>71</v>
       </c>
@@ -4605,7 +4837,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A73">
         <v>72</v>
       </c>
@@ -4646,7 +4878,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A74">
         <v>73</v>
       </c>
@@ -4688,7 +4920,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A75">
         <v>74</v>
       </c>
@@ -4727,7 +4959,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A76">
         <v>75</v>
       </c>
@@ -4766,7 +4998,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A77">
         <v>76</v>
       </c>
@@ -4806,7 +5038,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A78">
         <v>77</v>
       </c>
@@ -4844,7 +5076,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="79" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A79">
         <v>78</v>
       </c>
@@ -4883,7 +5115,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="80" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A80">
         <v>79</v>
       </c>
@@ -4922,7 +5154,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A81">
         <v>80</v>
       </c>
@@ -4960,12 +5192,12 @@
         <v>388</v>
       </c>
     </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A82">
         <v>81</v>
       </c>
       <c r="B82" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C82" t="s">
         <v>8</v>
@@ -4989,21 +5221,21 @@
         <v>3</v>
       </c>
       <c r="J82" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="K82">
         <v>9</v>
       </c>
       <c r="L82" s="1" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.25">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="83" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A83">
         <v>82</v>
       </c>
       <c r="B83" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="C83" t="s">
         <v>8</v>
@@ -5027,22 +5259,25 @@
         <v>7</v>
       </c>
       <c r="J83" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="K83">
         <f>I83*3</f>
         <v>21</v>
       </c>
       <c r="L83" s="1" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.25">
+        <v>394</v>
+      </c>
+      <c r="M83" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="84" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A84">
         <v>83</v>
       </c>
       <c r="B84" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="C84" t="s">
         <v>8</v>
@@ -5067,207 +5302,706 @@
         <v>2</v>
       </c>
       <c r="J84" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="K84">
         <f>6</f>
         <v>6</v>
       </c>
       <c r="L84" s="1" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.25">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="85" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A85">
         <v>84</v>
       </c>
+      <c r="B85" t="s">
+        <v>398</v>
+      </c>
       <c r="C85" t="s">
         <v>8</v>
       </c>
       <c r="D85" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E85" t="s">
+        <v>122</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+      <c r="G85" t="s">
+        <v>11</v>
+      </c>
+      <c r="H85" t="s">
+        <v>39</v>
+      </c>
+      <c r="I85">
+        <v>4</v>
+      </c>
+      <c r="J85" t="s">
+        <v>399</v>
+      </c>
+      <c r="K85">
+        <f>4*I85</f>
+        <v>16</v>
+      </c>
+      <c r="L85" s="1" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="86" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A86">
         <v>85</v>
       </c>
+      <c r="B86" t="s">
+        <v>402</v>
+      </c>
       <c r="C86" t="s">
         <v>8</v>
       </c>
       <c r="D86" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E86" t="s">
+        <v>33</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+      <c r="G86" t="s">
+        <v>382</v>
+      </c>
+      <c r="H86" t="s">
+        <v>383</v>
+      </c>
+      <c r="I86">
+        <v>8</v>
+      </c>
+      <c r="J86" t="s">
+        <v>401</v>
+      </c>
+      <c r="K86">
+        <f>8*4</f>
+        <v>32</v>
+      </c>
+      <c r="L86" s="1" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="87" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A87">
         <v>86</v>
       </c>
+      <c r="B87" t="s">
+        <v>404</v>
+      </c>
       <c r="C87" t="s">
         <v>8</v>
       </c>
       <c r="D87" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E87" t="s">
+        <v>50</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+      <c r="G87" t="s">
+        <v>11</v>
+      </c>
+      <c r="H87" t="s">
+        <v>407</v>
+      </c>
+      <c r="I87">
+        <v>4</v>
+      </c>
+      <c r="J87" t="s">
+        <v>406</v>
+      </c>
+      <c r="K87">
+        <f>4*4</f>
+        <v>16</v>
+      </c>
+      <c r="L87" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="M87" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="88" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A88">
         <v>87</v>
       </c>
+      <c r="B88" t="s">
+        <v>409</v>
+      </c>
       <c r="C88" t="s">
         <v>8</v>
       </c>
       <c r="D88" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E88" t="s">
+        <v>50</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+      <c r="G88" t="s">
+        <v>18</v>
+      </c>
+      <c r="H88" t="s">
+        <v>39</v>
+      </c>
+      <c r="I88">
+        <v>4</v>
+      </c>
+      <c r="J88" t="s">
+        <v>410</v>
+      </c>
+      <c r="K88">
+        <f>4*5</f>
+        <v>20</v>
+      </c>
+      <c r="L88" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="N88" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="89" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A89">
         <v>88</v>
       </c>
+      <c r="B89" t="s">
+        <v>419</v>
+      </c>
       <c r="C89" t="s">
         <v>8</v>
       </c>
       <c r="D89" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E89" t="s">
+        <v>122</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+      <c r="G89" t="s">
+        <v>420</v>
+      </c>
+      <c r="H89" t="s">
+        <v>421</v>
+      </c>
+      <c r="I89">
+        <v>6</v>
+      </c>
+      <c r="J89" t="s">
+        <v>422</v>
+      </c>
+      <c r="K89">
+        <f>6*3</f>
+        <v>18</v>
+      </c>
+      <c r="L89" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="M89" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="90" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A90">
         <v>89</v>
       </c>
+      <c r="B90" t="s">
+        <v>426</v>
+      </c>
       <c r="C90" t="s">
         <v>8</v>
       </c>
       <c r="D90" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E90" t="s">
+        <v>50</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+      <c r="G90" t="s">
+        <v>11</v>
+      </c>
+      <c r="H90" t="s">
+        <v>39</v>
+      </c>
+      <c r="I90">
+        <v>3</v>
+      </c>
+      <c r="J90" t="s">
+        <v>427</v>
+      </c>
+      <c r="K90">
+        <f>3*4</f>
+        <v>12</v>
+      </c>
+      <c r="L90" s="1" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="91" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A91">
         <v>90</v>
       </c>
+      <c r="B91" t="s">
+        <v>429</v>
+      </c>
       <c r="C91" t="s">
         <v>8</v>
       </c>
       <c r="D91" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E91" t="s">
+        <v>122</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+      <c r="G91" t="s">
+        <v>430</v>
+      </c>
+      <c r="H91" t="s">
+        <v>431</v>
+      </c>
+      <c r="I91">
+        <v>3</v>
+      </c>
+      <c r="J91" t="s">
+        <v>432</v>
+      </c>
+      <c r="K91">
+        <f>6</f>
+        <v>6</v>
+      </c>
+      <c r="L91" s="1" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="92" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A92">
         <v>91</v>
       </c>
+      <c r="B92" t="s">
+        <v>436</v>
+      </c>
       <c r="C92" t="s">
         <v>8</v>
       </c>
       <c r="D92" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E92" t="s">
+        <v>67</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+      <c r="G92" t="s">
+        <v>11</v>
+      </c>
+      <c r="H92" t="s">
+        <v>435</v>
+      </c>
+      <c r="I92">
+        <v>3</v>
+      </c>
+      <c r="J92" t="s">
+        <v>434</v>
+      </c>
+      <c r="K92">
+        <v>13</v>
+      </c>
+      <c r="L92" s="1" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="93" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A93">
         <v>92</v>
       </c>
+      <c r="B93" t="s">
+        <v>438</v>
+      </c>
       <c r="C93" t="s">
         <v>8</v>
       </c>
       <c r="D93" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E93" t="s">
+        <v>12</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+      <c r="G93" t="s">
+        <v>11</v>
+      </c>
+      <c r="H93" t="s">
+        <v>39</v>
+      </c>
+      <c r="I93">
+        <v>4</v>
+      </c>
+      <c r="J93" t="s">
+        <v>439</v>
+      </c>
+      <c r="K93">
+        <f>158</f>
+        <v>158</v>
+      </c>
+      <c r="L93" s="1" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="94" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A94">
         <v>93</v>
       </c>
+      <c r="B94" t="s">
+        <v>441</v>
+      </c>
       <c r="C94" t="s">
         <v>8</v>
       </c>
       <c r="D94" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E94" t="s">
+        <v>122</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+      <c r="G94" t="s">
+        <v>341</v>
+      </c>
+      <c r="H94" t="s">
+        <v>442</v>
+      </c>
+      <c r="I94">
+        <v>2</v>
+      </c>
+      <c r="J94" t="s">
+        <v>443</v>
+      </c>
+      <c r="K94">
+        <f>16</f>
+        <v>16</v>
+      </c>
+      <c r="L94" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="M94" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="95" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A95">
         <v>94</v>
       </c>
+      <c r="B95" t="s">
+        <v>445</v>
+      </c>
       <c r="C95" t="s">
         <v>8</v>
       </c>
       <c r="D95" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E95" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+      <c r="G95" t="s">
+        <v>447</v>
+      </c>
+      <c r="H95" t="s">
+        <v>39</v>
+      </c>
+      <c r="I95">
+        <v>2</v>
+      </c>
+      <c r="J95" t="s">
+        <v>446</v>
+      </c>
+      <c r="K95">
+        <v>6</v>
+      </c>
+      <c r="L95" t="s">
+        <v>47</v>
+      </c>
+      <c r="M95" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="96" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A96">
         <v>95</v>
       </c>
+      <c r="B96" s="5" t="s">
+        <v>448</v>
+      </c>
       <c r="C96" t="s">
         <v>8</v>
       </c>
       <c r="D96" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E96" t="s">
+        <v>122</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+      <c r="G96" t="s">
+        <v>18</v>
+      </c>
+      <c r="H96" t="s">
+        <v>450</v>
+      </c>
+      <c r="I96">
+        <v>6</v>
+      </c>
+      <c r="J96" t="s">
+        <v>449</v>
+      </c>
+      <c r="K96">
+        <f>6*8</f>
+        <v>48</v>
+      </c>
+      <c r="L96" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="M96" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="97" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A97">
         <v>96</v>
       </c>
+      <c r="B97" t="s">
+        <v>452</v>
+      </c>
       <c r="C97" t="s">
         <v>8</v>
       </c>
       <c r="D97" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E97" t="s">
+        <v>45</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+      <c r="G97" t="s">
+        <v>430</v>
+      </c>
+      <c r="H97" t="s">
+        <v>39</v>
+      </c>
+      <c r="I97">
+        <v>4</v>
+      </c>
+      <c r="J97" t="s">
+        <v>453</v>
+      </c>
+      <c r="K97">
+        <f>4*3</f>
+        <v>12</v>
+      </c>
+      <c r="L97" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="M97" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="98" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A98">
         <v>97</v>
       </c>
+      <c r="B98" t="s">
+        <v>454</v>
+      </c>
       <c r="C98" t="s">
         <v>8</v>
       </c>
       <c r="D98" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E98" t="s">
+        <v>211</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+      <c r="G98" t="s">
+        <v>11</v>
+      </c>
+      <c r="H98" t="s">
+        <v>57</v>
+      </c>
+      <c r="I98">
+        <v>3</v>
+      </c>
+      <c r="J98" t="s">
+        <v>455</v>
+      </c>
+      <c r="K98">
+        <f>30</f>
+        <v>30</v>
+      </c>
+      <c r="L98" s="1" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="99" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A99">
         <v>98</v>
       </c>
+      <c r="B99" t="s">
+        <v>459</v>
+      </c>
       <c r="C99" t="s">
         <v>8</v>
       </c>
       <c r="D99" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E99" t="s">
+        <v>460</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+      <c r="G99" t="s">
+        <v>11</v>
+      </c>
+      <c r="H99" t="s">
+        <v>57</v>
+      </c>
+      <c r="I99">
+        <v>3</v>
+      </c>
+      <c r="J99" t="s">
+        <v>458</v>
+      </c>
+      <c r="K99">
+        <f>15</f>
+        <v>15</v>
+      </c>
+      <c r="L99" s="1" t="s">
+        <v>461</v>
+      </c>
+      <c r="M99" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="100" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A100">
         <v>99</v>
       </c>
+      <c r="B100" t="s">
+        <v>463</v>
+      </c>
       <c r="C100" t="s">
         <v>8</v>
       </c>
       <c r="D100" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E100" t="s">
+        <v>31</v>
+      </c>
+      <c r="F100" t="s">
+        <v>56</v>
+      </c>
+      <c r="G100" t="s">
+        <v>464</v>
+      </c>
+      <c r="H100" t="s">
+        <v>115</v>
+      </c>
+      <c r="I100">
+        <v>3</v>
+      </c>
+      <c r="J100" t="s">
+        <v>462</v>
+      </c>
+      <c r="K100">
+        <f>60</f>
+        <v>60</v>
+      </c>
+      <c r="L100" t="s">
+        <v>47</v>
+      </c>
+      <c r="M100" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="101" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A101">
         <v>100</v>
       </c>
+      <c r="B101" t="s">
+        <v>466</v>
+      </c>
       <c r="C101" t="s">
         <v>8</v>
       </c>
       <c r="D101" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B102" t="s">
-        <v>389</v>
-      </c>
+      <c r="E101" t="s">
+        <v>67</v>
+      </c>
+      <c r="F101" t="s">
+        <v>56</v>
+      </c>
+      <c r="G101" t="s">
+        <v>18</v>
+      </c>
+      <c r="H101" t="s">
+        <v>77</v>
+      </c>
+      <c r="I101">
+        <v>3</v>
+      </c>
+      <c r="J101" t="s">
+        <v>465</v>
+      </c>
+      <c r="K101">
+        <f>3*4</f>
+        <v>12</v>
+      </c>
+      <c r="L101" s="1" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="102" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="B102" s="1"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:N81" xr:uid="{8BCF4AC8-88B5-4543-8C52-FD30450BEA57}"/>
@@ -5341,18 +6075,33 @@
     <hyperlink ref="L82" r:id="rId67" xr:uid="{2274C7CE-0848-479C-8E48-A92AFCD2DAF3}"/>
     <hyperlink ref="L83" r:id="rId68" tooltip="Persistent link using digital object identifier" xr:uid="{27BFC4E4-9DCB-4C1D-B672-888C8D8E2732}"/>
     <hyperlink ref="L84" r:id="rId69" xr:uid="{3593983D-93B4-45AC-8DAA-EEEB7814C6DA}"/>
+    <hyperlink ref="L85" r:id="rId70" xr:uid="{EC9CC085-AE00-427A-8A98-D6B7FAC40915}"/>
+    <hyperlink ref="L86" r:id="rId71" xr:uid="{37B11193-AEED-49A8-8DC8-B8B1A4B50E16}"/>
+    <hyperlink ref="L87" r:id="rId72" xr:uid="{A403A46C-980D-45D5-B1F3-6B41994824E5}"/>
+    <hyperlink ref="L88" r:id="rId73" xr:uid="{15C15D05-2BF6-429B-990B-D4D122B2135A}"/>
+    <hyperlink ref="L89" r:id="rId74" display="https://pubs.acs.org/doi/abs/10.1021/acs.jproteome.6b00211" xr:uid="{C8CA3592-D189-4484-9578-3CE6AA7AAAF0}"/>
+    <hyperlink ref="L90" r:id="rId75" xr:uid="{EA5E6D9D-EB0C-4CD0-A732-5E51418702BE}"/>
+    <hyperlink ref="L91" r:id="rId76" display="https://doi.org/10.1016/j.jbc.2021.100408" xr:uid="{B898DC3E-877C-48D3-B8DB-38527442C91C}"/>
+    <hyperlink ref="L92" r:id="rId77" xr:uid="{E631AF55-B593-4564-AD7B-C50AA064B385}"/>
+    <hyperlink ref="L93" r:id="rId78" xr:uid="{B2B70E0C-93B6-4E11-96C1-A5E9EACBC9AA}"/>
+    <hyperlink ref="L94" r:id="rId79" xr:uid="{9AE33C66-89B4-4F2A-8E68-CFB244668468}"/>
+    <hyperlink ref="L96" r:id="rId80" xr:uid="{DE49CA08-17FF-4C18-8C19-DF135E909D8E}"/>
+    <hyperlink ref="L98" r:id="rId81" xr:uid="{8925AE44-1384-4094-9B9F-CDCD372A1CA9}"/>
+    <hyperlink ref="L97" r:id="rId82" xr:uid="{69516E89-6753-4063-B3E0-FCDA495C291D}"/>
+    <hyperlink ref="L99" r:id="rId83" xr:uid="{58BA4A32-0915-4B17-956C-DBF2AC5940FA}"/>
+    <hyperlink ref="L101" r:id="rId84" xr:uid="{74804044-9702-465A-B0D4-A230294D0CE5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId70"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId85"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F2087B5-F5A7-4715-8903-807F8D9032AE}">
   <dimension ref="A1:O2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:15" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" s="2" customFormat="1" ht="15.9" x14ac:dyDescent="0.45">
       <c r="A1" s="2" t="s">
         <v>43</v>
       </c>
@@ -5399,7 +6148,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>15</v>
       </c>
@@ -5456,13 +6205,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5412E459-6599-4D39-A6E4-9FCCBAA2B3FA}">
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="65.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="65.53515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -5470,7 +6219,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>251</v>
       </c>
@@ -5478,7 +6227,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>254</v>
       </c>
@@ -5486,7 +6235,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>256</v>
       </c>
@@ -5494,7 +6243,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>258</v>
       </c>
@@ -5502,7 +6251,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>315</v>
       </c>
@@ -5510,12 +6259,44 @@
         <v>320</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>339</v>
       </c>
       <c r="B7" t="s">
         <v>345</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A8" t="s">
+        <v>413</v>
+      </c>
+      <c r="B8" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A9" t="s">
+        <v>415</v>
+      </c>
+      <c r="B9" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A10" t="s">
+        <v>417</v>
+      </c>
+      <c r="B10" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A11" t="s">
+        <v>424</v>
+      </c>
+      <c r="B11" t="s">
+        <v>425</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Final database with datasets included for gold standard
</commit_message>
<xml_diff>
--- a/goldStandard/_Index.xlsx
+++ b/goldStandard/_Index.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julia\Documents\GitHub\normScore\goldStandard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE5062FE-6E5A-460F-8B06-332CF3AFEA76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97648E71-C17B-4B4C-A4FD-8AE0DC5F8736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19320" yWindow="-2745" windowWidth="19440" windowHeight="14880" xr2:uid="{F827C457-048B-4104-BF2A-59E43A6422D6}"/>
+    <workbookView xWindow="16260" yWindow="2340" windowWidth="38700" windowHeight="15240" xr2:uid="{F827C457-048B-4104-BF2A-59E43A6422D6}"/>
   </bookViews>
   <sheets>
     <sheet name="In" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Possible" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">In!$A$1:$N$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">In!$A$1:$N$101</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1028" uniqueCount="476">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1030" uniqueCount="478">
   <si>
     <t>ID</t>
   </si>
@@ -932,9 +932,6 @@
     <t>Table from publication with group information</t>
   </si>
   <si>
-    <t>XLSX: PXD015422_44321_2021_BFEMMM202013257_MOESM2_ESM.xlsx</t>
-  </si>
-  <si>
     <t>PXD020722.2</t>
   </si>
   <si>
@@ -1340,9 +1337,6 @@
     <t>T-cell</t>
   </si>
   <si>
-    <t> PXD030132</t>
-  </si>
-  <si>
     <t>DOI: 10.1016/J.CELL.2025.06.023</t>
   </si>
   <si>
@@ -1458,6 +1452,18 @@
   </si>
   <si>
     <t>PXD022038_Conditionsassessed.xlsx</t>
+  </si>
+  <si>
+    <t>PXD030132</t>
+  </si>
+  <si>
+    <t>XLSX: PXD020722_44321_2021_BFEMMM202013257_MOESM2_ESM.xlsx</t>
+  </si>
+  <si>
+    <t>PXD015422</t>
+  </si>
+  <si>
+    <t>PXD020722  aparecia con ese identificador, por si acaso no futuro hai problemas con estes datasets</t>
   </si>
 </sst>
 </file>
@@ -1537,13 +1543,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -1871,20 +1876,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BCF4AC8-88B5-4543-8C52-FD30450BEA57}">
   <dimension ref="A1:N102"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="13.3046875" customWidth="1"/>
-    <col min="5" max="5" width="22.84375" customWidth="1"/>
-    <col min="6" max="6" width="15.3046875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.69140625" customWidth="1"/>
-    <col min="8" max="8" width="27.84375" customWidth="1"/>
-    <col min="10" max="10" width="14.3046875" customWidth="1"/>
-    <col min="12" max="12" width="38.3046875" customWidth="1"/>
-    <col min="13" max="13" width="40.69140625" customWidth="1"/>
-    <col min="14" max="14" width="38.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" customWidth="1"/>
+    <col min="5" max="5" width="22.85546875" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.7109375" customWidth="1"/>
+    <col min="8" max="8" width="27.85546875" customWidth="1"/>
+    <col min="10" max="10" width="149.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="38.28515625" customWidth="1"/>
+    <col min="13" max="13" width="40.7109375" customWidth="1"/>
+    <col min="14" max="14" width="38.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="2" customFormat="1" ht="15.9" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:14" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>43</v>
       </c>
@@ -1928,7 +1933,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1973,7 +1978,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2015,7 +2020,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2052,7 +2057,7 @@
       </c>
       <c r="M4" s="1"/>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2091,7 +2096,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2135,7 +2140,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2180,7 +2185,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2223,7 +2228,7 @@
       </c>
       <c r="N8" s="4"/>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2268,7 +2273,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2309,7 +2314,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2350,7 +2355,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2389,7 +2394,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2430,7 +2435,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2472,7 +2477,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2513,7 +2518,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2551,7 +2556,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -2589,7 +2594,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -2627,7 +2632,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2669,7 +2674,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -2710,7 +2715,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -2752,7 +2757,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -2794,7 +2799,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -2836,7 +2841,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -2876,7 +2881,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -2914,7 +2919,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -2952,7 +2957,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -2991,7 +2996,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -3030,7 +3035,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -3069,7 +3074,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -3108,7 +3113,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -3147,7 +3152,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -3189,7 +3194,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -3229,7 +3234,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -3268,7 +3273,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -3307,7 +3312,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -3346,7 +3351,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -3391,7 +3396,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -3430,7 +3435,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -3469,7 +3474,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -3511,7 +3516,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -3556,7 +3561,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -3598,7 +3603,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -3640,7 +3645,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -3681,7 +3686,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -3722,7 +3727,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -3764,7 +3769,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -3805,7 +3810,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -3843,7 +3848,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
@@ -3885,7 +3890,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
@@ -3928,7 +3933,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
@@ -3971,7 +3976,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
@@ -4012,7 +4017,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
@@ -4056,7 +4061,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
@@ -4098,7 +4103,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>54</v>
       </c>
@@ -4140,7 +4145,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
@@ -4182,7 +4187,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>56</v>
       </c>
@@ -4224,7 +4229,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
@@ -4265,7 +4270,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>58</v>
       </c>
@@ -4306,7 +4311,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>59</v>
       </c>
@@ -4347,7 +4352,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
@@ -4376,7 +4381,7 @@
         <v>4</v>
       </c>
       <c r="J61" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="K61">
         <f>63+52</f>
@@ -4386,18 +4391,18 @@
         <v>298</v>
       </c>
       <c r="M61" t="s">
-        <v>300</v>
+        <v>475</v>
       </c>
       <c r="N61" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C62" t="s">
         <v>8</v>
@@ -4421,7 +4426,7 @@
         <v>4</v>
       </c>
       <c r="J62" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="K62">
         <f>120</f>
@@ -4431,15 +4436,15 @@
         <v>298</v>
       </c>
       <c r="M62" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.4">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C63" t="s">
         <v>8</v>
@@ -4463,24 +4468,24 @@
         <v>6</v>
       </c>
       <c r="J63" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="K63">
         <v>36</v>
       </c>
       <c r="L63" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="M63" t="s">
         <v>305</v>
       </c>
-      <c r="M63" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.4">
+    </row>
+    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C64" t="s">
         <v>8</v>
@@ -4504,24 +4509,24 @@
         <v>5</v>
       </c>
       <c r="J64" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="K64">
         <v>35</v>
       </c>
       <c r="L64" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="M64" t="s">
         <v>309</v>
       </c>
-      <c r="M64" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.4">
+    </row>
+    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C65" t="s">
         <v>8</v>
@@ -4536,7 +4541,7 @@
         <v>273</v>
       </c>
       <c r="G65" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H65" t="s">
         <v>57</v>
@@ -4545,7 +4550,7 @@
         <v>3</v>
       </c>
       <c r="J65" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="K65">
         <v>9</v>
@@ -4554,15 +4559,15 @@
         <v>47</v>
       </c>
       <c r="N65" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.4">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>65</v>
       </c>
       <c r="B66" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C66" t="s">
         <v>8</v>
@@ -4580,28 +4585,28 @@
         <v>18</v>
       </c>
       <c r="H66" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="I66">
         <v>6</v>
       </c>
       <c r="J66" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="K66">
         <f>I66*3</f>
         <v>18</v>
       </c>
       <c r="L66" s="1" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.4">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C67" t="s">
         <v>8</v>
@@ -4625,7 +4630,7 @@
         <v>2</v>
       </c>
       <c r="J67" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="K67">
         <f>12</f>
@@ -4635,15 +4640,15 @@
         <v>47</v>
       </c>
       <c r="M67" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.4">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>67</v>
       </c>
       <c r="B68" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C68" t="s">
         <v>8</v>
@@ -4658,30 +4663,30 @@
         <v>9</v>
       </c>
       <c r="G68" t="s">
+        <v>324</v>
+      </c>
+      <c r="H68" t="s">
         <v>325</v>
-      </c>
-      <c r="H68" t="s">
-        <v>326</v>
       </c>
       <c r="I68">
         <v>2</v>
       </c>
       <c r="J68" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="K68">
         <v>12</v>
       </c>
       <c r="L68" s="1" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.4">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C69" t="s">
         <v>8</v>
@@ -4693,7 +4698,7 @@
         <v>33</v>
       </c>
       <c r="F69" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="G69" t="s">
         <v>11</v>
@@ -4705,22 +4710,22 @@
         <v>2</v>
       </c>
       <c r="J69" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="K69">
         <f>6</f>
         <v>6</v>
       </c>
       <c r="L69" s="1" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.4">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="70" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C70" t="s">
         <v>8</v>
@@ -4729,13 +4734,13 @@
         <v>99</v>
       </c>
       <c r="E70" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="F70" t="s">
         <v>131</v>
       </c>
       <c r="G70" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H70" t="s">
         <v>234</v>
@@ -4744,24 +4749,24 @@
         <v>2</v>
       </c>
       <c r="J70" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="K70">
         <v>10</v>
       </c>
       <c r="L70" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="N70" t="s">
         <v>343</v>
       </c>
-      <c r="N70" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.4">
+    </row>
+    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C71" t="s">
         <v>8</v>
@@ -4770,40 +4775,40 @@
         <v>99</v>
       </c>
       <c r="E71" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="F71" t="s">
         <v>131</v>
       </c>
       <c r="G71" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H71" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="I71">
         <v>5</v>
       </c>
       <c r="J71" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="K71">
         <f>I71*4+4</f>
         <v>24</v>
       </c>
       <c r="L71" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="N71" t="s">
         <v>350</v>
       </c>
-      <c r="N71" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.4">
+    </row>
+    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C72" t="s">
         <v>8</v>
@@ -4818,31 +4823,31 @@
         <v>131</v>
       </c>
       <c r="G72" t="s">
+        <v>353</v>
+      </c>
+      <c r="H72" t="s">
         <v>354</v>
-      </c>
-      <c r="H72" t="s">
-        <v>355</v>
       </c>
       <c r="I72">
         <v>3</v>
       </c>
       <c r="J72" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="K72">
         <f>3*4</f>
         <v>12</v>
       </c>
       <c r="L72" s="1" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.4">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>72</v>
       </c>
       <c r="B73" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C73" t="s">
         <v>8</v>
@@ -4851,7 +4856,7 @@
         <v>98</v>
       </c>
       <c r="E73" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F73" t="s">
         <v>9</v>
@@ -4860,30 +4865,30 @@
         <v>11</v>
       </c>
       <c r="H73" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="I73">
         <v>4</v>
       </c>
       <c r="J73" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="K73">
         <v>23</v>
       </c>
       <c r="L73" s="1" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="M73" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.4">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>73</v>
       </c>
       <c r="B74" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="C74" t="s">
         <v>8</v>
@@ -4898,34 +4903,34 @@
         <v>9</v>
       </c>
       <c r="G74" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H74" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="I74">
         <v>12</v>
       </c>
       <c r="J74" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="K74">
         <f>I74*6</f>
         <v>72</v>
       </c>
       <c r="L74" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="M74" t="s">
         <v>360</v>
       </c>
-      <c r="M74" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.4">
+    </row>
+    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>74</v>
       </c>
       <c r="B75" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C75" t="s">
         <v>8</v>
@@ -4940,7 +4945,7 @@
         <v>9</v>
       </c>
       <c r="G75" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H75" t="s">
         <v>136</v>
@@ -4949,22 +4954,22 @@
         <v>6</v>
       </c>
       <c r="J75" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="K75">
         <f>6*3</f>
         <v>18</v>
       </c>
       <c r="L75" s="1" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.4">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>75</v>
       </c>
       <c r="B76" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C76" t="s">
         <v>8</v>
@@ -4973,37 +4978,37 @@
         <v>98</v>
       </c>
       <c r="E76" t="s">
+        <v>365</v>
+      </c>
+      <c r="F76" t="s">
         <v>366</v>
       </c>
-      <c r="F76" t="s">
+      <c r="G76" t="s">
+        <v>324</v>
+      </c>
+      <c r="H76" t="s">
         <v>367</v>
-      </c>
-      <c r="G76" t="s">
-        <v>325</v>
-      </c>
-      <c r="H76" t="s">
-        <v>368</v>
       </c>
       <c r="I76">
         <v>3</v>
       </c>
       <c r="J76" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="K76">
         <f>I76*3</f>
         <v>9</v>
       </c>
       <c r="L76" s="1" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.4">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>76</v>
       </c>
       <c r="B77" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C77" t="s">
         <v>8</v>
@@ -5018,32 +5023,32 @@
         <v>9</v>
       </c>
       <c r="G77" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="H77" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="I77">
         <f>3</f>
         <v>3</v>
       </c>
       <c r="J77" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="K77">
         <f>I77*3</f>
         <v>9</v>
       </c>
       <c r="L77" s="1" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.4">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="78" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>77</v>
       </c>
       <c r="B78" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C78" t="s">
         <v>8</v>
@@ -5067,21 +5072,21 @@
         <v>2</v>
       </c>
       <c r="J78" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="K78">
         <v>15</v>
       </c>
       <c r="L78" s="1" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="79" spans="1:14" x14ac:dyDescent="0.4">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="79" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>78</v>
       </c>
       <c r="B79" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C79" t="s">
         <v>8</v>
@@ -5099,28 +5104,28 @@
         <v>18</v>
       </c>
       <c r="H79" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="I79">
         <v>3</v>
       </c>
       <c r="J79" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="K79">
         <f>9</f>
         <v>9</v>
       </c>
       <c r="L79" s="1" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="80" spans="1:14" x14ac:dyDescent="0.4">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="80" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>79</v>
       </c>
       <c r="B80" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C80" t="s">
         <v>8</v>
@@ -5135,31 +5140,31 @@
         <v>9</v>
       </c>
       <c r="G80" t="s">
+        <v>381</v>
+      </c>
+      <c r="H80" t="s">
         <v>382</v>
-      </c>
-      <c r="H80" t="s">
-        <v>383</v>
       </c>
       <c r="I80">
         <v>2</v>
       </c>
       <c r="J80" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="K80">
         <f>6</f>
         <v>6</v>
       </c>
       <c r="L80" s="1" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.4">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="81" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>80</v>
       </c>
       <c r="B81" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C81" t="s">
         <v>8</v>
@@ -5189,15 +5194,15 @@
         <v>6</v>
       </c>
       <c r="L81" s="1" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="82" spans="1:14" x14ac:dyDescent="0.4">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>81</v>
       </c>
       <c r="B82" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C82" t="s">
         <v>8</v>
@@ -5215,27 +5220,27 @@
         <v>18</v>
       </c>
       <c r="H82" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="I82">
         <v>3</v>
       </c>
       <c r="J82" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="K82">
         <v>9</v>
       </c>
       <c r="L82" s="1" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="83" spans="1:14" x14ac:dyDescent="0.4">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>82</v>
       </c>
       <c r="B83" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C83" t="s">
         <v>8</v>
@@ -5259,25 +5264,25 @@
         <v>7</v>
       </c>
       <c r="J83" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="K83">
         <f>I83*3</f>
         <v>21</v>
       </c>
       <c r="L83" s="1" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="M83" t="s">
-        <v>475</v>
-      </c>
-    </row>
-    <row r="84" spans="1:14" x14ac:dyDescent="0.4">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="84" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>83</v>
       </c>
       <c r="B84" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C84" t="s">
         <v>8</v>
@@ -5292,7 +5297,7 @@
         <v>9</v>
       </c>
       <c r="G84" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H84" t="s">
         <v>39</v>
@@ -5302,22 +5307,22 @@
         <v>2</v>
       </c>
       <c r="J84" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="K84">
         <f>6</f>
         <v>6</v>
       </c>
       <c r="L84" s="1" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="85" spans="1:14" x14ac:dyDescent="0.4">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="85" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>84</v>
       </c>
       <c r="B85" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C85" t="s">
         <v>8</v>
@@ -5341,22 +5346,22 @@
         <v>4</v>
       </c>
       <c r="J85" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="K85">
         <f>4*I85</f>
         <v>16</v>
       </c>
       <c r="L85" s="1" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.4">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="86" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>85</v>
       </c>
       <c r="B86" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C86" t="s">
         <v>8</v>
@@ -5371,31 +5376,31 @@
         <v>9</v>
       </c>
       <c r="G86" t="s">
+        <v>381</v>
+      </c>
+      <c r="H86" t="s">
         <v>382</v>
       </c>
-      <c r="H86" t="s">
-        <v>383</v>
-      </c>
       <c r="I86">
         <v>8</v>
       </c>
       <c r="J86" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="K86">
         <f>8*4</f>
         <v>32</v>
       </c>
       <c r="L86" s="1" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="87" spans="1:14" x14ac:dyDescent="0.4">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="87" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>86</v>
       </c>
       <c r="B87" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C87" t="s">
         <v>8</v>
@@ -5413,31 +5418,31 @@
         <v>11</v>
       </c>
       <c r="H87" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="I87">
         <v>4</v>
       </c>
       <c r="J87" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="K87">
         <f>4*4</f>
         <v>16</v>
       </c>
       <c r="L87" s="1" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="M87" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="88" spans="1:14" x14ac:dyDescent="0.4">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="88" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>87</v>
       </c>
       <c r="B88" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C88" t="s">
         <v>8</v>
@@ -5461,25 +5466,25 @@
         <v>4</v>
       </c>
       <c r="J88" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="K88">
         <f>4*5</f>
         <v>20</v>
       </c>
       <c r="L88" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="N88" t="s">
         <v>411</v>
       </c>
-      <c r="N88" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="89" spans="1:14" x14ac:dyDescent="0.4">
+    </row>
+    <row r="89" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>88</v>
       </c>
       <c r="B89" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="C89" t="s">
         <v>8</v>
@@ -5494,34 +5499,34 @@
         <v>9</v>
       </c>
       <c r="G89" t="s">
+        <v>419</v>
+      </c>
+      <c r="H89" t="s">
         <v>420</v>
-      </c>
-      <c r="H89" t="s">
-        <v>421</v>
       </c>
       <c r="I89">
         <v>6</v>
       </c>
       <c r="J89" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="K89">
         <f>6*3</f>
         <v>18</v>
       </c>
       <c r="L89" s="1" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="M89" t="s">
-        <v>474</v>
-      </c>
-    </row>
-    <row r="90" spans="1:14" x14ac:dyDescent="0.4">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="90" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>89</v>
       </c>
       <c r="B90" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C90" t="s">
         <v>8</v>
@@ -5545,22 +5550,22 @@
         <v>3</v>
       </c>
       <c r="J90" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="K90">
         <f>3*4</f>
         <v>12</v>
       </c>
       <c r="L90" s="1" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="91" spans="1:14" x14ac:dyDescent="0.4">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="91" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>90</v>
       </c>
       <c r="B91" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C91" t="s">
         <v>8</v>
@@ -5575,31 +5580,31 @@
         <v>9</v>
       </c>
       <c r="G91" t="s">
+        <v>429</v>
+      </c>
+      <c r="H91" t="s">
         <v>430</v>
-      </c>
-      <c r="H91" t="s">
-        <v>431</v>
       </c>
       <c r="I91">
         <v>3</v>
       </c>
       <c r="J91" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="K91">
         <f>6</f>
         <v>6</v>
       </c>
       <c r="L91" s="1" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="92" spans="1:14" x14ac:dyDescent="0.4">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="92" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>91</v>
       </c>
       <c r="B92" t="s">
-        <v>436</v>
+        <v>474</v>
       </c>
       <c r="C92" t="s">
         <v>8</v>
@@ -5617,27 +5622,27 @@
         <v>11</v>
       </c>
       <c r="H92" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="I92">
         <v>3</v>
       </c>
       <c r="J92" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="K92">
         <v>13</v>
       </c>
       <c r="L92" s="1" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="93" spans="1:14" x14ac:dyDescent="0.4">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="93" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>92</v>
       </c>
       <c r="B93" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="C93" t="s">
         <v>8</v>
@@ -5661,22 +5666,22 @@
         <v>4</v>
       </c>
       <c r="J93" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="K93">
         <f>158</f>
         <v>158</v>
       </c>
       <c r="L93" s="1" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="94" spans="1:14" x14ac:dyDescent="0.4">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="94" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>93</v>
       </c>
       <c r="B94" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="C94" t="s">
         <v>8</v>
@@ -5691,34 +5696,34 @@
         <v>9</v>
       </c>
       <c r="G94" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H94" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="I94">
         <v>2</v>
       </c>
       <c r="J94" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="K94">
         <f>16</f>
         <v>16</v>
       </c>
       <c r="L94" s="1" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="M94" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="95" spans="1:14" x14ac:dyDescent="0.4">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="95" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>94</v>
       </c>
       <c r="B95" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="C95" t="s">
         <v>8</v>
@@ -5726,14 +5731,14 @@
       <c r="D95" t="s">
         <v>98</v>
       </c>
-      <c r="E95" s="5" t="s">
+      <c r="E95" t="s">
         <v>50</v>
       </c>
       <c r="F95" t="s">
         <v>9</v>
       </c>
       <c r="G95" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="H95" t="s">
         <v>39</v>
@@ -5742,7 +5747,7 @@
         <v>2</v>
       </c>
       <c r="J95" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="K95">
         <v>6</v>
@@ -5751,15 +5756,15 @@
         <v>47</v>
       </c>
       <c r="M95" t="s">
-        <v>472</v>
-      </c>
-    </row>
-    <row r="96" spans="1:14" x14ac:dyDescent="0.4">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="96" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>95</v>
       </c>
-      <c r="B96" s="5" t="s">
-        <v>448</v>
+      <c r="B96" t="s">
+        <v>446</v>
       </c>
       <c r="C96" t="s">
         <v>8</v>
@@ -5777,31 +5782,31 @@
         <v>18</v>
       </c>
       <c r="H96" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="I96">
         <v>6</v>
       </c>
       <c r="J96" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="K96">
         <f>6*8</f>
         <v>48</v>
       </c>
       <c r="L96" s="1" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="M96" t="s">
-        <v>471</v>
-      </c>
-    </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.4">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="97" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>96</v>
       </c>
       <c r="B97" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="C97" t="s">
         <v>8</v>
@@ -5816,7 +5821,7 @@
         <v>9</v>
       </c>
       <c r="G97" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="H97" t="s">
         <v>39</v>
@@ -5825,25 +5830,25 @@
         <v>4</v>
       </c>
       <c r="J97" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="K97">
         <f>4*3</f>
         <v>12</v>
       </c>
       <c r="L97" s="1" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="M97" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="98" spans="1:13" x14ac:dyDescent="0.4">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="98" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>97</v>
       </c>
       <c r="B98" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="C98" t="s">
         <v>8</v>
@@ -5867,22 +5872,22 @@
         <v>3</v>
       </c>
       <c r="J98" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="K98">
         <f>30</f>
         <v>30</v>
       </c>
       <c r="L98" s="1" t="s">
-        <v>456</v>
-      </c>
-    </row>
-    <row r="99" spans="1:13" x14ac:dyDescent="0.4">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="99" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>98</v>
       </c>
       <c r="B99" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="C99" t="s">
         <v>8</v>
@@ -5891,7 +5896,7 @@
         <v>98</v>
       </c>
       <c r="E99" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="F99" t="s">
         <v>9</v>
@@ -5906,25 +5911,25 @@
         <v>3</v>
       </c>
       <c r="J99" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="K99">
         <f>15</f>
         <v>15</v>
       </c>
       <c r="L99" s="1" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="M99" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="100" spans="1:13" x14ac:dyDescent="0.4">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="100" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>99</v>
       </c>
       <c r="B100" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="C100" t="s">
         <v>8</v>
@@ -5939,7 +5944,7 @@
         <v>56</v>
       </c>
       <c r="G100" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="H100" t="s">
         <v>115</v>
@@ -5948,7 +5953,7 @@
         <v>3</v>
       </c>
       <c r="J100" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="K100">
         <f>60</f>
@@ -5958,15 +5963,15 @@
         <v>47</v>
       </c>
       <c r="M100" t="s">
-        <v>468</v>
-      </c>
-    </row>
-    <row r="101" spans="1:13" x14ac:dyDescent="0.4">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="101" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>100</v>
       </c>
       <c r="B101" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="C101" t="s">
         <v>8</v>
@@ -5990,21 +5995,21 @@
         <v>3</v>
       </c>
       <c r="J101" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="K101">
         <f>3*4</f>
         <v>12</v>
       </c>
       <c r="L101" s="1" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="102" spans="1:13" x14ac:dyDescent="0.4">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="102" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B102" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N81" xr:uid="{8BCF4AC8-88B5-4543-8C52-FD30450BEA57}"/>
+  <autoFilter ref="A1:N101" xr:uid="{8BCF4AC8-88B5-4543-8C52-FD30450BEA57}"/>
   <hyperlinks>
     <hyperlink ref="L4" r:id="rId1" display="https://doi.org/10.1016/j.stemcr.2022.04.003" xr:uid="{A58B2C92-8135-4993-80B6-E01F7C4414D7}"/>
     <hyperlink ref="L2" r:id="rId2" xr:uid="{ECF580C4-849C-4561-A481-5430106E5AFC}"/>
@@ -6099,9 +6104,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F2087B5-F5A7-4715-8903-807F8D9032AE}">
   <dimension ref="A1:O2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:15" s="2" customFormat="1" ht="15.9" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:15" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>43</v>
       </c>
@@ -6148,7 +6153,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>15</v>
       </c>
@@ -6205,13 +6210,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5412E459-6599-4D39-A6E4-9FCCBAA2B3FA}">
-  <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="65.53515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="65.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -6219,7 +6224,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>251</v>
       </c>
@@ -6227,7 +6232,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>254</v>
       </c>
@@ -6235,7 +6240,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>256</v>
       </c>
@@ -6243,7 +6248,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>258</v>
       </c>
@@ -6251,52 +6256,60 @@
         <v>259</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B6" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B7" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>412</v>
+      </c>
+      <c r="B8" t="s">
         <v>413</v>
       </c>
-      <c r="B8" t="s">
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>414</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A9" t="s">
+      <c r="B9" t="s">
         <v>415</v>
       </c>
-      <c r="B9" t="s">
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>416</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A10" t="s">
+      <c r="B10" t="s">
         <v>417</v>
       </c>
-      <c r="B10" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>423</v>
+      </c>
+      <c r="B11" t="s">
         <v>424</v>
       </c>
-      <c r="B11" t="s">
-        <v>425</v>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>476</v>
+      </c>
+      <c r="B12" t="s">
+        <v>477</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated index xlsx file
</commit_message>
<xml_diff>
--- a/goldStandard/_Index.xlsx
+++ b/goldStandard/_Index.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julia\Documents\GitHub\normScore-development\goldStandard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB851249-1EA9-41A9-BDBA-C9A7AC4626CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCC13A02-D14B-45E8-8F5E-5FEA36084C63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10485" yWindow="4200" windowWidth="37380" windowHeight="12765" xr2:uid="{F827C457-048B-4104-BF2A-59E43A6422D6}"/>
+    <workbookView xWindow="930" yWindow="1065" windowWidth="29700" windowHeight="19665" xr2:uid="{F827C457-048B-4104-BF2A-59E43A6422D6}"/>
   </bookViews>
   <sheets>
     <sheet name="In" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1475" uniqueCount="718">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1475" uniqueCount="716">
   <si>
     <t>ID</t>
   </si>
@@ -2175,16 +2175,10 @@
     <t>MS instrument (summary)</t>
   </si>
   <si>
-    <t>Orbitrap</t>
-  </si>
-  <si>
-    <t>Orbitrap;Q Exactive</t>
-  </si>
-  <si>
-    <t>TripleTOF</t>
-  </si>
-  <si>
-    <t>ZenoTOF</t>
+    <t>TOF-based</t>
+  </si>
+  <si>
+    <t>Orbitrap-based</t>
   </si>
 </sst>
 </file>
@@ -2692,7 +2686,7 @@
         <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F2" t="s">
         <v>9</v>
@@ -2752,7 +2746,7 @@
         <v>105</v>
       </c>
       <c r="E3" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F3" t="s">
         <v>9</v>
@@ -2808,7 +2802,7 @@
         <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F4" t="s">
         <v>9</v>
@@ -2860,7 +2854,7 @@
         <v>29</v>
       </c>
       <c r="E5" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F5" t="s">
         <v>9</v>
@@ -2914,7 +2908,7 @@
         <v>33</v>
       </c>
       <c r="E6" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F6" t="s">
         <v>9</v>
@@ -2970,7 +2964,7 @@
         <v>39</v>
       </c>
       <c r="E7" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F7" t="s">
         <v>9</v>
@@ -3027,7 +3021,7 @@
         <v>43</v>
       </c>
       <c r="E8" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F8" t="s">
         <v>9</v>
@@ -3082,7 +3076,7 @@
         <v>12</v>
       </c>
       <c r="E9" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F9" t="s">
         <v>48</v>
@@ -3139,7 +3133,7 @@
         <v>53</v>
       </c>
       <c r="E10" t="s">
-        <v>315</v>
+        <v>714</v>
       </c>
       <c r="F10" t="s">
         <v>48</v>
@@ -3192,7 +3186,7 @@
         <v>57</v>
       </c>
       <c r="E11" t="s">
-        <v>315</v>
+        <v>714</v>
       </c>
       <c r="F11" t="s">
         <v>48</v>
@@ -3245,7 +3239,7 @@
         <v>61</v>
       </c>
       <c r="E12" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F12" t="s">
         <v>48</v>
@@ -3296,7 +3290,7 @@
         <v>27</v>
       </c>
       <c r="E13" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F13" t="s">
         <v>9</v>
@@ -3349,7 +3343,7 @@
         <v>43</v>
       </c>
       <c r="E14" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F14" t="s">
         <v>9</v>
@@ -3403,7 +3397,7 @@
         <v>57</v>
       </c>
       <c r="E15" t="s">
-        <v>315</v>
+        <v>714</v>
       </c>
       <c r="F15" t="s">
         <v>9</v>
@@ -3506,7 +3500,7 @@
         <v>27</v>
       </c>
       <c r="E17" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F17" t="s">
         <v>9</v>
@@ -3556,7 +3550,7 @@
         <v>61</v>
       </c>
       <c r="E18" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F18" t="s">
         <v>9</v>
@@ -3609,7 +3603,7 @@
         <v>27</v>
       </c>
       <c r="E19" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F19" t="s">
         <v>9</v>
@@ -3663,7 +3657,7 @@
         <v>105</v>
       </c>
       <c r="E20" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F20" t="s">
         <v>9</v>
@@ -3719,7 +3713,7 @@
         <v>29</v>
       </c>
       <c r="E21" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F21" t="s">
         <v>9</v>
@@ -3773,7 +3767,7 @@
         <v>111</v>
       </c>
       <c r="E22" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="F22" t="s">
         <v>112</v>
@@ -3827,7 +3821,7 @@
         <v>105</v>
       </c>
       <c r="E23" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F23" t="s">
         <v>112</v>
@@ -3881,7 +3875,7 @@
         <v>43</v>
       </c>
       <c r="E24" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F24" t="s">
         <v>112</v>
@@ -3932,7 +3926,7 @@
         <v>122</v>
       </c>
       <c r="E25" t="s">
-        <v>315</v>
+        <v>714</v>
       </c>
       <c r="F25" t="s">
         <v>112</v>
@@ -3982,7 +3976,7 @@
         <v>53</v>
       </c>
       <c r="E26" t="s">
-        <v>315</v>
+        <v>714</v>
       </c>
       <c r="F26" t="s">
         <v>112</v>
@@ -4032,7 +4026,7 @@
         <v>39</v>
       </c>
       <c r="E27" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F27" t="s">
         <v>112</v>
@@ -4083,7 +4077,7 @@
         <v>105</v>
       </c>
       <c r="E28" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F28" t="s">
         <v>112</v>
@@ -4133,7 +4127,7 @@
         <v>57</v>
       </c>
       <c r="E29" t="s">
-        <v>315</v>
+        <v>714</v>
       </c>
       <c r="F29" t="s">
         <v>112</v>
@@ -4184,7 +4178,7 @@
         <v>134</v>
       </c>
       <c r="E30" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F30" t="s">
         <v>112</v>
@@ -4235,7 +4229,7 @@
         <v>139</v>
       </c>
       <c r="E31" t="s">
-        <v>139</v>
+        <v>714</v>
       </c>
       <c r="F31" t="s">
         <v>112</v>
@@ -4253,13 +4247,12 @@
         <v>475</v>
       </c>
       <c r="K31">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L31" t="s">
         <v>140</v>
       </c>
       <c r="M31">
-        <f>K31*4</f>
         <v>16</v>
       </c>
       <c r="N31" s="1" t="s">
@@ -4286,7 +4279,7 @@
         <v>57</v>
       </c>
       <c r="E32" t="s">
-        <v>315</v>
+        <v>714</v>
       </c>
       <c r="F32" t="s">
         <v>112</v>
@@ -4340,7 +4333,7 @@
         <v>151</v>
       </c>
       <c r="E33" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F33" t="s">
         <v>112</v>
@@ -4392,7 +4385,7 @@
         <v>27</v>
       </c>
       <c r="E34" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F34" t="s">
         <v>112</v>
@@ -4410,7 +4403,7 @@
         <v>478</v>
       </c>
       <c r="K34">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L34" t="s">
         <v>156</v>
@@ -4443,7 +4436,7 @@
         <v>12</v>
       </c>
       <c r="E35" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F35" t="s">
         <v>112</v>
@@ -4494,7 +4487,7 @@
         <v>164</v>
       </c>
       <c r="E36" t="s">
-        <v>315</v>
+        <v>714</v>
       </c>
       <c r="F36" t="s">
         <v>112</v>
@@ -4545,7 +4538,7 @@
         <v>61</v>
       </c>
       <c r="E37" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F37" t="s">
         <v>112</v>
@@ -4602,7 +4595,7 @@
         <v>27</v>
       </c>
       <c r="E38" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F38" t="s">
         <v>112</v>
@@ -4653,7 +4646,7 @@
         <v>172</v>
       </c>
       <c r="E39" t="s">
-        <v>315</v>
+        <v>714</v>
       </c>
       <c r="F39" t="s">
         <v>112</v>
@@ -4704,7 +4697,7 @@
         <v>53</v>
       </c>
       <c r="E40" t="s">
-        <v>315</v>
+        <v>714</v>
       </c>
       <c r="F40" t="s">
         <v>112</v>
@@ -4758,7 +4751,7 @@
         <v>57</v>
       </c>
       <c r="E41" t="s">
-        <v>315</v>
+        <v>714</v>
       </c>
       <c r="F41" t="s">
         <v>112</v>
@@ -4815,7 +4808,7 @@
         <v>105</v>
       </c>
       <c r="E42" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F42" t="s">
         <v>9</v>
@@ -4869,7 +4862,7 @@
         <v>186</v>
       </c>
       <c r="E43" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="F43" t="s">
         <v>112</v>
@@ -4923,7 +4916,7 @@
         <v>18</v>
       </c>
       <c r="E44" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F44" t="s">
         <v>112</v>
@@ -4976,7 +4969,7 @@
         <v>18</v>
       </c>
       <c r="E45" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F45" t="s">
         <v>112</v>
@@ -5029,7 +5022,7 @@
         <v>111</v>
       </c>
       <c r="E46" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="F46" t="s">
         <v>112</v>
@@ -5047,7 +5040,7 @@
         <v>489</v>
       </c>
       <c r="K46">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L46" t="s">
         <v>590</v>
@@ -5083,7 +5076,7 @@
         <v>18</v>
       </c>
       <c r="E47" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F47" t="s">
         <v>112</v>
@@ -5136,7 +5129,7 @@
         <v>207</v>
       </c>
       <c r="E48" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F48" t="s">
         <v>112</v>
@@ -5186,7 +5179,7 @@
         <v>39</v>
       </c>
       <c r="E49" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F49" t="s">
         <v>112</v>
@@ -5240,7 +5233,7 @@
         <v>18</v>
       </c>
       <c r="E50" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F50" t="s">
         <v>112</v>
@@ -5295,7 +5288,7 @@
         <v>111</v>
       </c>
       <c r="E51" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="F51" t="s">
         <v>112</v>
@@ -5350,7 +5343,7 @@
         <v>18</v>
       </c>
       <c r="E52" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F52" t="s">
         <v>112</v>
@@ -5403,7 +5396,7 @@
         <v>186</v>
       </c>
       <c r="E53" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="F53" t="s">
         <v>235</v>
@@ -5459,7 +5452,7 @@
         <v>39</v>
       </c>
       <c r="E54" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F54" t="s">
         <v>112</v>
@@ -5513,7 +5506,7 @@
         <v>151</v>
       </c>
       <c r="E55" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F55" t="s">
         <v>246</v>
@@ -5567,7 +5560,7 @@
         <v>43</v>
       </c>
       <c r="E56" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F56" t="s">
         <v>246</v>
@@ -5621,7 +5614,7 @@
         <v>105</v>
       </c>
       <c r="E57" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F57" t="s">
         <v>246</v>
@@ -5675,7 +5668,7 @@
         <v>43</v>
       </c>
       <c r="E58" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F58" t="s">
         <v>246</v>
@@ -5728,7 +5721,7 @@
         <v>39</v>
       </c>
       <c r="E59" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F59" t="s">
         <v>246</v>
@@ -5781,7 +5774,7 @@
         <v>27</v>
       </c>
       <c r="E60" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F60" t="s">
         <v>246</v>
@@ -5834,7 +5827,7 @@
         <v>43</v>
       </c>
       <c r="E61" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F61" t="s">
         <v>246</v>
@@ -5891,7 +5884,7 @@
         <v>43</v>
       </c>
       <c r="E62" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F62" t="s">
         <v>246</v>
@@ -5945,7 +5938,7 @@
         <v>39</v>
       </c>
       <c r="E63" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F63" t="s">
         <v>246</v>
@@ -5998,7 +5991,7 @@
         <v>39</v>
       </c>
       <c r="E64" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F64" t="s">
         <v>112</v>
@@ -6051,7 +6044,7 @@
         <v>43</v>
       </c>
       <c r="E65" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F65" t="s">
         <v>246</v>
@@ -6107,7 +6100,7 @@
         <v>43</v>
       </c>
       <c r="E66" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F66" t="s">
         <v>246</v>
@@ -6161,7 +6154,7 @@
         <v>57</v>
       </c>
       <c r="E67" t="s">
-        <v>315</v>
+        <v>714</v>
       </c>
       <c r="F67" t="s">
         <v>246</v>
@@ -6218,7 +6211,7 @@
         <v>57</v>
       </c>
       <c r="E68" t="s">
-        <v>315</v>
+        <v>714</v>
       </c>
       <c r="F68" t="s">
         <v>9</v>
@@ -6268,7 +6261,7 @@
         <v>29</v>
       </c>
       <c r="E69" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F69" t="s">
         <v>299</v>
@@ -6319,7 +6312,7 @@
         <v>308</v>
       </c>
       <c r="E70" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="F70" t="s">
         <v>112</v>
@@ -6372,7 +6365,7 @@
         <v>315</v>
       </c>
       <c r="E71" t="s">
-        <v>315</v>
+        <v>714</v>
       </c>
       <c r="F71" t="s">
         <v>112</v>
@@ -6426,7 +6419,7 @@
         <v>18</v>
       </c>
       <c r="E72" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F72" t="s">
         <v>112</v>
@@ -6477,7 +6470,7 @@
         <v>305</v>
       </c>
       <c r="E73" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F73" t="s">
         <v>9</v>
@@ -6530,7 +6523,7 @@
         <v>105</v>
       </c>
       <c r="E74" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F74" t="s">
         <v>9</v>
@@ -6584,7 +6577,7 @@
         <v>105</v>
       </c>
       <c r="E75" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F75" t="s">
         <v>9</v>
@@ -6635,7 +6628,7 @@
         <v>334</v>
       </c>
       <c r="E76" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F76" t="s">
         <v>9</v>
@@ -6686,7 +6679,7 @@
         <v>29</v>
       </c>
       <c r="E77" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F77" t="s">
         <v>9</v>
@@ -6738,7 +6731,7 @@
         <v>27</v>
       </c>
       <c r="E78" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F78" t="s">
         <v>9</v>
@@ -6788,7 +6781,7 @@
         <v>43</v>
       </c>
       <c r="E79" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F79" t="s">
         <v>9</v>
@@ -6839,7 +6832,7 @@
         <v>29</v>
       </c>
       <c r="E80" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F80" t="s">
         <v>9</v>
@@ -6890,7 +6883,7 @@
         <v>29</v>
       </c>
       <c r="E81" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F81" t="s">
         <v>9</v>
@@ -6940,7 +6933,7 @@
         <v>43</v>
       </c>
       <c r="E82" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F82" t="s">
         <v>9</v>
@@ -6990,7 +6983,7 @@
         <v>105</v>
       </c>
       <c r="E83" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F83" t="s">
         <v>9</v>
@@ -7044,7 +7037,7 @@
         <v>105</v>
       </c>
       <c r="E84" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F84" t="s">
         <v>9</v>
@@ -7096,7 +7089,7 @@
         <v>105</v>
       </c>
       <c r="E85" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F85" t="s">
         <v>9</v>
@@ -7147,7 +7140,7 @@
         <v>29</v>
       </c>
       <c r="E86" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F86" t="s">
         <v>9</v>
@@ -7198,7 +7191,7 @@
         <v>43</v>
       </c>
       <c r="E87" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F87" t="s">
         <v>9</v>
@@ -7252,7 +7245,7 @@
         <v>43</v>
       </c>
       <c r="E88" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F88" t="s">
         <v>9</v>
@@ -7306,7 +7299,7 @@
         <v>105</v>
       </c>
       <c r="E89" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F89" t="s">
         <v>9</v>
@@ -7324,7 +7317,7 @@
         <v>386</v>
       </c>
       <c r="K89">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L89" t="s">
         <v>387</v>
@@ -7360,7 +7353,7 @@
         <v>43</v>
       </c>
       <c r="E90" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F90" t="s">
         <v>9</v>
@@ -7411,7 +7404,7 @@
         <v>105</v>
       </c>
       <c r="E91" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F91" t="s">
         <v>9</v>
@@ -7429,7 +7422,7 @@
         <v>396</v>
       </c>
       <c r="K91">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L91" t="s">
         <v>397</v>
@@ -7462,7 +7455,7 @@
         <v>57</v>
       </c>
       <c r="E92" t="s">
-        <v>315</v>
+        <v>714</v>
       </c>
       <c r="F92" t="s">
         <v>9</v>
@@ -7512,7 +7505,7 @@
         <v>12</v>
       </c>
       <c r="E93" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F93" t="s">
         <v>9</v>
@@ -7563,7 +7556,7 @@
         <v>105</v>
       </c>
       <c r="E94" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F94" t="s">
         <v>9</v>
@@ -7617,7 +7610,7 @@
         <v>43</v>
       </c>
       <c r="E95" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F95" t="s">
         <v>9</v>
@@ -7670,7 +7663,7 @@
         <v>105</v>
       </c>
       <c r="E96" t="s">
-        <v>105</v>
+        <v>715</v>
       </c>
       <c r="F96" t="s">
         <v>9</v>
@@ -7724,7 +7717,7 @@
         <v>39</v>
       </c>
       <c r="E97" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F97" t="s">
         <v>9</v>
@@ -7778,7 +7771,7 @@
         <v>186</v>
       </c>
       <c r="E98" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="F98" t="s">
         <v>9</v>
@@ -7829,7 +7822,7 @@
         <v>424</v>
       </c>
       <c r="E99" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F99" t="s">
         <v>9</v>
@@ -7883,7 +7876,7 @@
         <v>27</v>
       </c>
       <c r="E100" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F100" t="s">
         <v>48</v>
@@ -7937,7 +7930,7 @@
         <v>57</v>
       </c>
       <c r="E101" t="s">
-        <v>315</v>
+        <v>714</v>
       </c>
       <c r="F101" t="s">
         <v>48</v>

</xml_diff>

<commit_message>
Descriptive summary of GS manual asssessment
</commit_message>
<xml_diff>
--- a/goldStandard/_Index.xlsx
+++ b/goldStandard/_Index.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julia\Documents\GitHub\normScore-development\goldStandard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCC13A02-D14B-45E8-8F5E-5FEA36084C63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9220C87C-FFFA-48F0-BA5E-EAC8A76FB1FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="930" yWindow="1065" windowWidth="29700" windowHeight="19665" xr2:uid="{F827C457-048B-4104-BF2A-59E43A6422D6}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="15240" windowHeight="19365" xr2:uid="{F827C457-048B-4104-BF2A-59E43A6422D6}"/>
   </bookViews>
   <sheets>
     <sheet name="In" sheetId="1" r:id="rId1"/>
@@ -3893,7 +3893,6 @@
         <v>478</v>
       </c>
       <c r="K24">
-        <f>2</f>
         <v>2</v>
       </c>
       <c r="L24" t="s">
@@ -4351,7 +4350,6 @@
         <v>483</v>
       </c>
       <c r="K33">
-        <f>3</f>
         <v>3</v>
       </c>
       <c r="L33" t="s">
@@ -5251,7 +5249,6 @@
         <v>215</v>
       </c>
       <c r="K50">
-        <f>6</f>
         <v>6</v>
       </c>
       <c r="L50" t="s">
@@ -5306,7 +5303,6 @@
         <v>489</v>
       </c>
       <c r="K51">
-        <f>2</f>
         <v>2</v>
       </c>
       <c r="L51" t="s">
@@ -6697,7 +6693,6 @@
         <v>339</v>
       </c>
       <c r="K77">
-        <f>3</f>
         <v>3</v>
       </c>
       <c r="L77" t="s">
@@ -7055,7 +7050,6 @@
         <v>497</v>
       </c>
       <c r="K84">
-        <f>2</f>
         <v>2</v>
       </c>
       <c r="L84" t="s">

</xml_diff>